<commit_message>
freelance: lista lunga di 31 nicchie con segnali, note di verifica e foglio Fonti
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNxVApXF9MzdDwSEC8TCy4
</commit_message>
<xml_diff>
--- a/freelance/griglia-nicchie.xlsx
+++ b/freelance/griglia-nicchie.xlsx
@@ -10,9 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteri" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista lunga" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$U$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$U$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +67,12 @@
       <color rgb="007C8A91"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -102,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,6 +146,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -734,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V65"/>
+  <dimension ref="A1:V75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -770,7 +779,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Una riga per nicchia. In blu le celle da compilare: stima di aziende target e di prezzo (con fonte), punteggi 1-5. 'Clienti per 1 M€' e 'Punteggio' si calcolano da soli. Le candidate A-C sono ipotesi iniziali, non ancora valutate: dati di mercato non verificati.</t>
+          <t>Una riga per nicchia (lista lunga, Fase 1). Il segnale è solo il punto di partenza: la colonna Note dice se è stato verificato in ricerca (stampa di settore, non fonti ufficiali) o se è solo un'ipotesi. In blu le celle da compilare nelle fasi 2-3: stima di aziende target e di prezzo (con fonte) e punteggi 1-5. 'Clienti per 1 M€' e 'Punteggio' si calcolano da soli.</t>
         </is>
       </c>
     </row>
@@ -920,28 +929,28 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
+    <row r="6" ht="92" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>A. Strumenti per la filiera della fibra (report di collaudo, documentazione)</t>
+          <t>NIS2: preparazione alla conformità per PMI fornitrici di soggetti critici</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Imprese di posa fibra e installatori</t>
+          <t>PMI in filiere critiche; consulenti e MSP come canale</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Incentivi / fondi</t>
+          <t>Obbligo di legge</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Piano Italia 1 Giga in ritardo (Domani, Segugio)</t>
+          <t>Noze; Agenda Digitale</t>
         </is>
       </c>
       <c r="F6" s="10" t="n"/>
@@ -969,20 +978,24 @@
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="46" customHeight="1">
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Notifica incidenti operativa dal 15/01/2026; misure di base con scadenze da ottobre 2026 per chi ha ricevuto la comunicazione ad aprile 2025. Mercato affollato di consulenti. Numero di imprese coinvolte non trovato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
       <c r="A7" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>B. Preparazione alla NIS2 per PMI fornitrici di soggetti critici</t>
+          <t>NIS2 per MSP e consulenti: piattaforma multi-cliente per gestire la conformità di più aziende</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>PMI in filiere critiche; consulenti e MSP come canale</t>
+          <t>MSP, studi di consulenza IT</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -992,7 +1005,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Scadenze ACN 2026 (Noze, Agenda Digitale)</t>
+          <t>Noze; Agenda Digitale</t>
         </is>
       </c>
       <c r="F7" s="10" t="n"/>
@@ -1020,30 +1033,34 @@
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Variante della precedente: vendi al canale, non alla PMI finale. Da confrontare con piattaforme esistenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
       <c r="A8" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>C. Strumenti di pianificazione e monitoraggio per piccoli operatori FWA</t>
+          <t>Cyber Resilience Act: gestione segnalazione vulnerabilità e fascicolo tecnico per produttori</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Piccoli provider wireless</t>
+          <t>Produttori di prodotti con elementi digitali (elettronica, IoT, macchine con software)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Altro</t>
+          <t>Obbligo di legge</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>FWA &gt;2,7 M di linee (AGCOM via Segugio)</t>
+          <t>Agenda Digitale; IPSOA</t>
         </is>
       </c>
       <c r="F8" s="10" t="n"/>
@@ -1071,16 +1088,36 @@
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U8" s="6" t="n"/>
-    </row>
-    <row r="9">
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Obbligo di segnalazione dall'11/09/2026 (preallarme in 24 ore); piena applicazione 11/12/2027; sanzioni fino a 15 M€ (stampa). Vantaggio tuo: medio-alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
       <c r="A9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Direttiva RED (cybersicurezza): assistente alla conformità EN 18031 per produttori di apparecchi radio/IoT</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Produttori e importatori di apparecchi radio e dispositivi connessi</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>TÜV SÜD; Yarix</t>
+        </is>
+      </c>
       <c r="F9" s="10" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="10" t="n"/>
@@ -1101,17 +1138,41 @@
         <f>IF(COUNT(K9:R9)=0,"",ROUND(SUMPRODUCT(K9:R9,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T9" s="6" t="n"/>
-      <c r="U9" s="6" t="n"/>
-    </row>
-    <row r="10">
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Applicabile dal 01/08/2025. Stato di armonizzazione degli standard discordante tra le fonti. Vantaggio tuo: alto (RF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
       <c r="A10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Regolamento Macchine 2023/1230: generatore di fascicolo tecnico e dichiarazione UE</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Costruttori di macchine (Lombardia è un polo)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Certifico; UCIMU</t>
+        </is>
+      </c>
       <c r="F10" s="10" t="n"/>
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="10" t="n"/>
@@ -1132,17 +1193,41 @@
         <f>IF(COUNT(K10:R10)=0,"",ROUND(SUMPRODUCT(K10:R10,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T10" s="6" t="n"/>
-      <c r="U10" s="6" t="n"/>
-    </row>
-    <row r="11">
+      <c r="T10" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Applicazione dal 20/01/2027; UCIMU chiede una proroga condizionata. Dettagli sulla documentazione tecnica non verificati.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
       <c r="A11" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>AI Act: inventario dei sistemi di IA e conformità agli obblighi di trasparenza (art. 50)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>PMI che usano o forniscono sistemi di IA</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Agenda Digitale; Noze</t>
+        </is>
+      </c>
       <c r="F11" s="10" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="10" t="n"/>
@@ -1163,17 +1248,41 @@
         <f>IF(COUNT(K11:R11)=0,"",ROUND(SUMPRODUCT(K11:R11,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T11" s="6" t="n"/>
-      <c r="U11" s="6" t="n"/>
-    </row>
-    <row r="12">
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Trasparenza dal 02/08/2026; alto rischio rinviato a dicembre 2027 / agosto 2028 (accordo provvisorio del 07/05/2026, da verificare in Gazzetta UE). Domanda specifica debole.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="92" customHeight="1">
       <c r="A12" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Trasparenza retributiva: annunci e report sul divario di genere</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Aziende con 100+ dipendenti, uffici HR</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>QuiFinanza; PartitaIVA.it</t>
+        </is>
+      </c>
       <c r="F12" s="10" t="n"/>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="10" t="n"/>
@@ -1194,17 +1303,41 @@
         <f>IF(COUNT(K12:R12)=0,"",ROUND(SUMPRODUCT(K12:R12,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T12" s="6" t="n"/>
-      <c r="U12" s="6" t="n"/>
-    </row>
-    <row r="13">
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Stato del decreto di recepimento discordante tra le fonti (D.Lgs. 96/2026?). Report annuale dal 07/06/2027 per 250+ dipendenti. Il target è piccolo: poche aziende con 100+ dipendenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="92" customHeight="1">
       <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>PPWR imballaggi: gestione dati e dichiarazioni di conformità</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Produttori e utilizzatori di imballaggi (Lombardia ha molti)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Assolombarda</t>
+        </is>
+      </c>
       <c r="F13" s="10" t="n"/>
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="10" t="n"/>
@@ -1225,17 +1358,41 @@
         <f>IF(COUNT(K13:R13)=0,"",ROUND(SUMPRODUCT(K13:R13,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T13" s="6" t="n"/>
-      <c r="U13" s="6" t="n"/>
-    </row>
-    <row r="14">
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Applicabile dal 12/08/2026; date di etichettatura discordanti (2026, 2027, 2028). Assolombarda ha attivato un desk dedicato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="92" customHeight="1">
       <c r="A14" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Passaporto digitale di prodotto: raccolta dati per batterie e tessile</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Produttori di batterie e tessile</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Bluestone PIM; PMI.it</t>
+        </is>
+      </c>
       <c r="F14" s="10" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="10" t="n"/>
@@ -1256,17 +1413,41 @@
         <f>IF(COUNT(K14:R14)=0,"",ROUND(SUMPRODUCT(K14:R14,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T14" s="6" t="n"/>
-      <c r="U14" s="6" t="n"/>
-    </row>
-    <row r="15">
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Batterie dal 18/02/2027; tessile non ancora definito. Dominato da grandi fornitori e dagli atti delegati.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="92" customHeight="1">
       <c r="A15" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Accessibilità digitale (EAA): audit e correzione per e-commerce</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>E-commerce italiani</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Agenda Digitale; Iubenda</t>
+        </is>
+      </c>
       <c r="F15" s="10" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="10" t="n"/>
@@ -1287,17 +1468,41 @@
         <f>IF(COUNT(K15:R15)=0,"",ROUND(SUMPRODUCT(K15:R15,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T15" s="6" t="n"/>
-      <c r="U15" s="6" t="n"/>
-    </row>
-    <row r="16">
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Obbligo dal 28/06/2025; piattaforma di segnalazione AgID dal 11/03/2026; sanzioni da verificare (nessun procedimento pubblico trovato a giugno 2026). Molti fornitori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="92" customHeight="1">
       <c r="A16" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Iperammortamento 2026: pratica per perizia asseverata, certificazione e comunicazioni al GSE</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Studi di ingegneria che firmano perizie; imprese manifatturiere</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Incentivi / fondi</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Agenda Digitale; Pasquale Pillitteri</t>
+        </is>
+      </c>
       <c r="F16" s="10" t="n"/>
       <c r="G16" s="6" t="n"/>
       <c r="H16" s="10" t="n"/>
@@ -1318,17 +1523,41 @@
         <f>IF(COUNT(K16:R16)=0,"",ROUND(SUMPRODUCT(K16:R16,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T16" s="6" t="n"/>
-      <c r="U16" s="6" t="n"/>
-    </row>
-    <row r="17">
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Piattaforma GSE dal 12/06/2026; comunicazione di completamento entro 15/11/2028. La perizia è di un ingegnere iscritto all'albo: collegato agli studi che stai contattando. Regole (soglie, SaaS) discordanti tra le fonti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="92" customHeight="1">
       <c r="A17" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Fibra ottica: report di collaudo e documentazione per imprese di posa</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Imprese di posa fibra e installatori</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Incentivi / fondi</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Domani</t>
+        </is>
+      </c>
       <c r="F17" s="10" t="n"/>
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="10" t="n"/>
@@ -1349,17 +1578,41 @@
         <f>IF(COUNT(K17:R17)=0,"",ROUND(SUMPRODUCT(K17:R17,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T17" s="6" t="n"/>
-      <c r="U17" s="6" t="n"/>
-    </row>
-    <row r="18">
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Piano Italia 1 Giga in ritardo: 250–700 mila civici potrebbero uscire dal Piano. Committenti con portali propri; strumenti degli OTDR con report già inclusi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="92" customHeight="1">
       <c r="A18" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Comunità energetiche: piattaforma di gestione per CER, condomini e comuni</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Promotori di CER, amministratori di condominio, comuni</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Incentivi / fondi</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>InfoBuild Energia</t>
+        </is>
+      </c>
       <c r="F18" s="10" t="n"/>
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="10" t="n"/>
@@ -1380,17 +1633,41 @@
         <f>IF(COUNT(K18:R18)=0,"",ROUND(SUMPRODUCT(K18:R18,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T18" s="6" t="n"/>
-      <c r="U18" s="6" t="n"/>
-    </row>
-    <row r="19">
+      <c r="T18" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U18" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Obiettivo di 15.000 CER a giugno 2026 probabilmente mancato; regole ancora instabili.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="92" customHeight="1">
       <c r="A19" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Diagnosi energetica obbligatoria: strumento per redigere e gestire le diagnosi</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Studi di ingegneria, ESCO, grandi imprese ed energivori</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Incentivi / fondi</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>da cercare</t>
+        </is>
+      </c>
       <c r="F19" s="10" t="n"/>
       <c r="G19" s="6" t="n"/>
       <c r="H19" s="10" t="n"/>
@@ -1411,17 +1688,41 @@
         <f>IF(COUNT(K19:R19)=0,"",ROUND(SUMPRODUCT(K19:R19,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T19" s="6" t="n"/>
-      <c r="U19" s="6" t="n"/>
-    </row>
-    <row r="20">
+      <c r="T19" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U19" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato. Obbligo ricorrente (ogni 4 anni per le imprese soggette). Da verificare sulle norme e sul mercato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="92" customHeight="1">
       <c r="A20" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>FWA: pianificazione e monitoraggio per piccoli operatori wireless</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Piccoli provider FWA/WISP</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Segugio (dati AGCOM)</t>
+        </is>
+      </c>
       <c r="F20" s="10" t="n"/>
       <c r="G20" s="6" t="n"/>
       <c r="H20" s="10" t="n"/>
@@ -1442,17 +1743,41 @@
         <f>IF(COUNT(K20:R20)=0,"",ROUND(SUMPRODUCT(K20:R20,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T20" s="6" t="n"/>
-      <c r="U20" s="6" t="n"/>
-    </row>
-    <row r="21">
+      <c r="T20" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U20" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Oltre 2,7 milioni di linee FWA, +13% in un anno; frequenze 26 GHz in assegnazione. Nessun dato recente sul numero di piccoli provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="92" customHeight="1">
       <c r="A21" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Audit e ottimizzazione dei costi telecom per PMI</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>PMI con molte linee e contratti</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>da cercare</t>
+        </is>
+      </c>
       <c r="F21" s="10" t="n"/>
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="10" t="n"/>
@@ -1473,17 +1798,41 @@
         <f>IF(COUNT(K21:R21)=0,"",ROUND(SUMPRODUCT(K21:R21,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T21" s="6" t="n"/>
-      <c r="U21" s="6" t="n"/>
-    </row>
-    <row r="22">
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U21" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Vantaggio tuo alto; modello a risparmio condiviso. Da verificare quanto si risparmia davvero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="92" customHeight="1">
       <c r="A22" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Pianificazione turni e presenze per magazzini, logistica e conto terzi</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Logistica, confezionamento conto terzi, magazzini</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Acquisizioni di verticali</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Aventis Advisors (Zucchetti)</t>
+        </is>
+      </c>
       <c r="F22" s="10" t="n"/>
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="10" t="n"/>
@@ -1504,17 +1853,41 @@
         <f>IF(COUNT(K22:R22)=0,"",ROUND(SUMPRODUCT(K22:R22,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T22" s="6" t="n"/>
-      <c r="U22" s="6" t="n"/>
-    </row>
-    <row r="23">
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
+          <t>Zucchetti ha acquisito la maggioranza di AWMS (personale per fabbriche e logistica): segnale che il verticale vale. In zona: 6 imprese di conto terzi nell'elenco. Software di turni già presenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="92" customHeight="1">
       <c r="A23" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Gestione commesse e avanzamento lavori per piccole imprese edili e impiantisti</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Imprese edili, impiantisti</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Acquisizioni di verticali</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Aventis Advisors (TeamSystem)</t>
+        </is>
+      </c>
       <c r="F23" s="10" t="n"/>
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="10" t="n"/>
@@ -1535,17 +1908,41 @@
         <f>IF(COUNT(K23:R23)=0,"",ROUND(SUMPRODUCT(K23:R23,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T23" s="6" t="n"/>
-      <c r="U23" s="6" t="n"/>
-    </row>
-    <row r="24">
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U23" s="6" t="inlineStr">
+        <is>
+          <t>TeamSystem ha fatto 7 acquisizioni nel comparto industria/costruzioni/real estate: segnale di valore del verticale. Mercato presidiato da gruppi grandi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="92" customHeight="1">
       <c r="A24" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Scadenzario obblighi di sicurezza sul lavoro (formazione, visite, DPI) per PMI</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>PMI manifatturiere e di servizi</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Acquisizioni di verticali</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Aventis Advisors (TeamSystem: legal, compliance, sicurezza)</t>
+        </is>
+      </c>
       <c r="F24" s="10" t="n"/>
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="10" t="n"/>
@@ -1566,17 +1963,41 @@
         <f>IF(COUNT(K24:R24)=0,"",ROUND(SUMPRODUCT(K24:R24,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T24" s="6" t="n"/>
-      <c r="U24" s="6" t="n"/>
-    </row>
-    <row r="25">
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U24" s="6" t="inlineStr">
+        <is>
+          <t>5 acquisizioni TeamSystem in legal/compliance/sicurezza. Prodotti già esistenti; da mappare i concorrenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="92" customHeight="1">
       <c r="A25" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Report di collaudo automatici da dati di misura per laboratori e officine</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Laboratori di prova, officine di precisione, assemblatori</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>idea precedente</t>
+        </is>
+      </c>
       <c r="F25" s="10" t="n"/>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="10" t="n"/>
@@ -1597,17 +2018,41 @@
         <f>IF(COUNT(K25:R25)=0,"",ROUND(SUMPRODUCT(K25:R25,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T25" s="6" t="n"/>
-      <c r="U25" s="6" t="n"/>
-    </row>
-    <row r="26">
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U25" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Gli strumenti hanno già software di report. Vantaggio tuo: alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="92" customHeight="1">
       <c r="A26" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Scadenzario tarature degli strumenti di misura (ISO 9001)</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Officine, laboratori, PMI certificate</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>idea precedente</t>
+        </is>
+      </c>
       <c r="F26" s="10" t="n"/>
       <c r="G26" s="6" t="n"/>
       <c r="H26" s="10" t="n"/>
@@ -1628,17 +2073,41 @@
         <f>IF(COUNT(K26:R26)=0,"",ROUND(SUMPRODUCT(K26:R26,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T26" s="6" t="n"/>
-      <c r="U26" s="6" t="n"/>
-    </row>
-    <row r="27">
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U26" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="92" customHeight="1">
       <c r="A27" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Preventivatore con codici articolo per distributori tecnici</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Distributori di bulloneria, acciai, plastiche, macchine utensili</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>idea precedente</t>
+        </is>
+      </c>
       <c r="F27" s="10" t="n"/>
       <c r="G27" s="6" t="n"/>
       <c r="H27" s="10" t="n"/>
@@ -1659,17 +2128,41 @@
         <f>IF(COUNT(K27:R27)=0,"",ROUND(SUMPRODUCT(K27:R27,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T27" s="6" t="n"/>
-      <c r="U27" s="6" t="n"/>
-    </row>
-    <row r="28">
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U27" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Probabile presenza di gestionali; da verificare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="92" customHeight="1">
       <c r="A28" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Estrazione dati da ordini, DDT e preventivi in PDF per il back-office</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>PMI con ufficio ordini</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Annunci di lavoro</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>da cercare</t>
+        </is>
+      </c>
       <c r="F28" s="10" t="n"/>
       <c r="G28" s="6" t="n"/>
       <c r="H28" s="10" t="n"/>
@@ -1690,17 +2183,41 @@
         <f>IF(COUNT(K28:R28)=0,"",ROUND(SUMPRODUCT(K28:R28,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T28" s="6" t="n"/>
-      <c r="U28" s="6" t="n"/>
-    </row>
-    <row r="29">
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U28" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato. Da cercare tra gli annunci per ruoli ripetitivi (ufficio ordini, data entry).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="92" customHeight="1">
       <c r="A29" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Assistente a documentazione tecnica per l'assistenza post-vendita dei costruttori di macchine</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Costruttori di macchine</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>idea Gemini</t>
+        </is>
+      </c>
       <c r="F29" s="10" t="n"/>
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="10" t="n"/>
@@ -1721,17 +2238,41 @@
         <f>IF(COUNT(K29:R29)=0,"",ROUND(SUMPRODUCT(K29:R29,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T29" s="6" t="n"/>
-      <c r="U29" s="6" t="n"/>
-    </row>
-    <row r="30">
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U29" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="92" customHeight="1">
       <c r="A30" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Automazione di relazioni, perizie e pratiche per studi tecnici</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Studi di ingegneria e professionisti</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>studi contattati</t>
+        </is>
+      </c>
       <c r="F30" s="10" t="n"/>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="10" t="n"/>
@@ -1752,17 +2293,41 @@
         <f>IF(COUNT(K30:R30)=0,"",ROUND(SUMPRODUCT(K30:R30,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T30" s="6" t="n"/>
-      <c r="U30" s="6" t="n"/>
-    </row>
-    <row r="31">
+      <c r="T30" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U30" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Gli studi (DEAL, Parodi, Lommano) fanno pratiche antincendio, certificazioni energetiche, perizie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="92" customHeight="1">
       <c r="A31" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Gestione dei file di misura RF e ottici per R&amp;D e produzione</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Laboratori R&amp;D e produzione elettronica</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>tuo campo</t>
+        </is>
+      </c>
       <c r="F31" s="10" t="n"/>
       <c r="G31" s="6" t="n"/>
       <c r="H31" s="10" t="n"/>
@@ -1783,17 +2348,41 @@
         <f>IF(COUNT(K31:R31)=0,"",ROUND(SUMPRODUCT(K31:R31,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T31" s="6" t="n"/>
-      <c r="U31" s="6" t="n"/>
-    </row>
-    <row r="32">
+      <c r="T31" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U31" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Vantaggio tuo: alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="92" customHeight="1">
       <c r="A32" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Schede di sicurezza e conformità CLP/REACH per chimica e gomma-plastica</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Aziende chimiche e della gomma-plastica</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>segmenti B2B (non verificati)</t>
+        </is>
+      </c>
       <c r="F32" s="10" t="n"/>
       <c r="G32" s="6" t="n"/>
       <c r="H32" s="10" t="n"/>
@@ -1814,17 +2403,41 @@
         <f>IF(COUNT(K32:R32)=0,"",ROUND(SUMPRODUCT(K32:R32,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T32" s="6" t="n"/>
-      <c r="U32" s="6" t="n"/>
-    </row>
-    <row r="33">
+      <c r="T32" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="92" customHeight="1">
       <c r="A33" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Documentazione elettronica di lotto (batch record) per piccole aziende farmaceutiche/CDMO</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Piccole aziende farmaceutiche e CDMO</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>segmenti B2B (non verificati)</t>
+        </is>
+      </c>
       <c r="F33" s="10" t="n"/>
       <c r="G33" s="6" t="n"/>
       <c r="H33" s="10" t="n"/>
@@ -1845,17 +2458,41 @@
         <f>IF(COUNT(K33:R33)=0,"",ROUND(SUMPRODUCT(K33:R33,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T33" s="6" t="n"/>
-      <c r="U33" s="6" t="n"/>
-    </row>
-    <row r="34">
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U33" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato. Barriera regolatoria alta (GMP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="92" customHeight="1">
       <c r="A34" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Formazione e simulazioni di phishing per PMI (obblighi di formazione NIS2)</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Noze; Agenda Digitale</t>
+        </is>
+      </c>
       <c r="F34" s="10" t="n"/>
       <c r="G34" s="6" t="n"/>
       <c r="H34" s="10" t="n"/>
@@ -1876,17 +2513,41 @@
         <f>IF(COUNT(K34:R34)=0,"",ROUND(SUMPRODUCT(K34:R34,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T34" s="6" t="n"/>
-      <c r="U34" s="6" t="n"/>
-    </row>
-    <row r="35">
+      <c r="T34" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U34" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Mercato affollato e a basso prezzo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="92" customHeight="1">
       <c r="A35" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Manutenzione predittiva a basso costo per macchine di PMI manifatturiere</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>PMI manifatturiere</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>idea nostra</t>
+        </is>
+      </c>
       <c r="F35" s="10" t="n"/>
       <c r="G35" s="6" t="n"/>
       <c r="H35" s="10" t="n"/>
@@ -1907,17 +2568,41 @@
         <f>IF(COUNT(K35:R35)=0,"",ROUND(SUMPRODUCT(K35:R35,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T35" s="6" t="n"/>
-      <c r="U35" s="6" t="n"/>
-    </row>
-    <row r="36">
+      <c r="T35" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U35" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Concorrenza forte (grandi fornitori).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="92" customHeight="1">
       <c r="A36" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Gestione documentale per sicurezza prodotti (GPSR) di importatori e venditori online</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Importatori e e-commerce di prodotti per consumatori</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>da cercare</t>
+        </is>
+      </c>
       <c r="F36" s="10" t="n"/>
       <c r="G36" s="6" t="n"/>
       <c r="H36" s="10" t="n"/>
@@ -1938,8 +2623,16 @@
         <f>IF(COUNT(K36:R36)=0,"",ROUND(SUMPRODUCT(K36:R36,K$4:R$4)/SUM(K$4:R$4),2))</f>
         <v/>
       </c>
-      <c r="T36" s="6" t="n"/>
-      <c r="U36" s="6" t="n"/>
+      <c r="T36" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="U36" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
@@ -2840,19 +3533,329 @@
       <c r="T65" s="6" t="n"/>
       <c r="U65" s="6" t="n"/>
     </row>
+    <row r="66">
+      <c r="A66" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="10" t="n"/>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="10" t="n"/>
+      <c r="I66" s="11">
+        <f>IF(H66&gt;0,ROUND(1000000/H66,0),"")</f>
+        <v/>
+      </c>
+      <c r="J66" s="6" t="n"/>
+      <c r="K66" s="6" t="n"/>
+      <c r="L66" s="6" t="n"/>
+      <c r="M66" s="6" t="n"/>
+      <c r="N66" s="6" t="n"/>
+      <c r="O66" s="6" t="n"/>
+      <c r="P66" s="6" t="n"/>
+      <c r="Q66" s="6" t="n"/>
+      <c r="R66" s="6" t="n"/>
+      <c r="S66" s="4">
+        <f>IF(COUNT(K66:R66)=0,"",ROUND(SUMPRODUCT(K66:R66,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T66" s="6" t="n"/>
+      <c r="U66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="10" t="n"/>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="10" t="n"/>
+      <c r="I67" s="11">
+        <f>IF(H67&gt;0,ROUND(1000000/H67,0),"")</f>
+        <v/>
+      </c>
+      <c r="J67" s="6" t="n"/>
+      <c r="K67" s="6" t="n"/>
+      <c r="L67" s="6" t="n"/>
+      <c r="M67" s="6" t="n"/>
+      <c r="N67" s="6" t="n"/>
+      <c r="O67" s="6" t="n"/>
+      <c r="P67" s="6" t="n"/>
+      <c r="Q67" s="6" t="n"/>
+      <c r="R67" s="6" t="n"/>
+      <c r="S67" s="4">
+        <f>IF(COUNT(K67:R67)=0,"",ROUND(SUMPRODUCT(K67:R67,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T67" s="6" t="n"/>
+      <c r="U67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="10" t="n"/>
+      <c r="G68" s="6" t="n"/>
+      <c r="H68" s="10" t="n"/>
+      <c r="I68" s="11">
+        <f>IF(H68&gt;0,ROUND(1000000/H68,0),"")</f>
+        <v/>
+      </c>
+      <c r="J68" s="6" t="n"/>
+      <c r="K68" s="6" t="n"/>
+      <c r="L68" s="6" t="n"/>
+      <c r="M68" s="6" t="n"/>
+      <c r="N68" s="6" t="n"/>
+      <c r="O68" s="6" t="n"/>
+      <c r="P68" s="6" t="n"/>
+      <c r="Q68" s="6" t="n"/>
+      <c r="R68" s="6" t="n"/>
+      <c r="S68" s="4">
+        <f>IF(COUNT(K68:R68)=0,"",ROUND(SUMPRODUCT(K68:R68,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T68" s="6" t="n"/>
+      <c r="U68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="6" t="n"/>
+      <c r="F69" s="10" t="n"/>
+      <c r="G69" s="6" t="n"/>
+      <c r="H69" s="10" t="n"/>
+      <c r="I69" s="11">
+        <f>IF(H69&gt;0,ROUND(1000000/H69,0),"")</f>
+        <v/>
+      </c>
+      <c r="J69" s="6" t="n"/>
+      <c r="K69" s="6" t="n"/>
+      <c r="L69" s="6" t="n"/>
+      <c r="M69" s="6" t="n"/>
+      <c r="N69" s="6" t="n"/>
+      <c r="O69" s="6" t="n"/>
+      <c r="P69" s="6" t="n"/>
+      <c r="Q69" s="6" t="n"/>
+      <c r="R69" s="6" t="n"/>
+      <c r="S69" s="4">
+        <f>IF(COUNT(K69:R69)=0,"",ROUND(SUMPRODUCT(K69:R69,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T69" s="6" t="n"/>
+      <c r="U69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="6" t="n"/>
+      <c r="F70" s="10" t="n"/>
+      <c r="G70" s="6" t="n"/>
+      <c r="H70" s="10" t="n"/>
+      <c r="I70" s="11">
+        <f>IF(H70&gt;0,ROUND(1000000/H70,0),"")</f>
+        <v/>
+      </c>
+      <c r="J70" s="6" t="n"/>
+      <c r="K70" s="6" t="n"/>
+      <c r="L70" s="6" t="n"/>
+      <c r="M70" s="6" t="n"/>
+      <c r="N70" s="6" t="n"/>
+      <c r="O70" s="6" t="n"/>
+      <c r="P70" s="6" t="n"/>
+      <c r="Q70" s="6" t="n"/>
+      <c r="R70" s="6" t="n"/>
+      <c r="S70" s="4">
+        <f>IF(COUNT(K70:R70)=0,"",ROUND(SUMPRODUCT(K70:R70,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T70" s="6" t="n"/>
+      <c r="U70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="6" t="n"/>
+      <c r="F71" s="10" t="n"/>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="10" t="n"/>
+      <c r="I71" s="11">
+        <f>IF(H71&gt;0,ROUND(1000000/H71,0),"")</f>
+        <v/>
+      </c>
+      <c r="J71" s="6" t="n"/>
+      <c r="K71" s="6" t="n"/>
+      <c r="L71" s="6" t="n"/>
+      <c r="M71" s="6" t="n"/>
+      <c r="N71" s="6" t="n"/>
+      <c r="O71" s="6" t="n"/>
+      <c r="P71" s="6" t="n"/>
+      <c r="Q71" s="6" t="n"/>
+      <c r="R71" s="6" t="n"/>
+      <c r="S71" s="4">
+        <f>IF(COUNT(K71:R71)=0,"",ROUND(SUMPRODUCT(K71:R71,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T71" s="6" t="n"/>
+      <c r="U71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="6" t="n"/>
+      <c r="E72" s="6" t="n"/>
+      <c r="F72" s="10" t="n"/>
+      <c r="G72" s="6" t="n"/>
+      <c r="H72" s="10" t="n"/>
+      <c r="I72" s="11">
+        <f>IF(H72&gt;0,ROUND(1000000/H72,0),"")</f>
+        <v/>
+      </c>
+      <c r="J72" s="6" t="n"/>
+      <c r="K72" s="6" t="n"/>
+      <c r="L72" s="6" t="n"/>
+      <c r="M72" s="6" t="n"/>
+      <c r="N72" s="6" t="n"/>
+      <c r="O72" s="6" t="n"/>
+      <c r="P72" s="6" t="n"/>
+      <c r="Q72" s="6" t="n"/>
+      <c r="R72" s="6" t="n"/>
+      <c r="S72" s="4">
+        <f>IF(COUNT(K72:R72)=0,"",ROUND(SUMPRODUCT(K72:R72,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T72" s="6" t="n"/>
+      <c r="U72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="B73" s="6" t="n"/>
+      <c r="C73" s="6" t="n"/>
+      <c r="D73" s="6" t="n"/>
+      <c r="E73" s="6" t="n"/>
+      <c r="F73" s="10" t="n"/>
+      <c r="G73" s="6" t="n"/>
+      <c r="H73" s="10" t="n"/>
+      <c r="I73" s="11">
+        <f>IF(H73&gt;0,ROUND(1000000/H73,0),"")</f>
+        <v/>
+      </c>
+      <c r="J73" s="6" t="n"/>
+      <c r="K73" s="6" t="n"/>
+      <c r="L73" s="6" t="n"/>
+      <c r="M73" s="6" t="n"/>
+      <c r="N73" s="6" t="n"/>
+      <c r="O73" s="6" t="n"/>
+      <c r="P73" s="6" t="n"/>
+      <c r="Q73" s="6" t="n"/>
+      <c r="R73" s="6" t="n"/>
+      <c r="S73" s="4">
+        <f>IF(COUNT(K73:R73)=0,"",ROUND(SUMPRODUCT(K73:R73,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T73" s="6" t="n"/>
+      <c r="U73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="B74" s="6" t="n"/>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
+      <c r="E74" s="6" t="n"/>
+      <c r="F74" s="10" t="n"/>
+      <c r="G74" s="6" t="n"/>
+      <c r="H74" s="10" t="n"/>
+      <c r="I74" s="11">
+        <f>IF(H74&gt;0,ROUND(1000000/H74,0),"")</f>
+        <v/>
+      </c>
+      <c r="J74" s="6" t="n"/>
+      <c r="K74" s="6" t="n"/>
+      <c r="L74" s="6" t="n"/>
+      <c r="M74" s="6" t="n"/>
+      <c r="N74" s="6" t="n"/>
+      <c r="O74" s="6" t="n"/>
+      <c r="P74" s="6" t="n"/>
+      <c r="Q74" s="6" t="n"/>
+      <c r="R74" s="6" t="n"/>
+      <c r="S74" s="4">
+        <f>IF(COUNT(K74:R74)=0,"",ROUND(SUMPRODUCT(K74:R74,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T74" s="6" t="n"/>
+      <c r="U74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
+      <c r="F75" s="10" t="n"/>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="10" t="n"/>
+      <c r="I75" s="11">
+        <f>IF(H75&gt;0,ROUND(1000000/H75,0),"")</f>
+        <v/>
+      </c>
+      <c r="J75" s="6" t="n"/>
+      <c r="K75" s="6" t="n"/>
+      <c r="L75" s="6" t="n"/>
+      <c r="M75" s="6" t="n"/>
+      <c r="N75" s="6" t="n"/>
+      <c r="O75" s="6" t="n"/>
+      <c r="P75" s="6" t="n"/>
+      <c r="Q75" s="6" t="n"/>
+      <c r="R75" s="6" t="n"/>
+      <c r="S75" s="4">
+        <f>IF(COUNT(K75:R75)=0,"",ROUND(SUMPRODUCT(K75:R75,K$4:R$4)/SUM(K$4:R$4),2))</f>
+        <v/>
+      </c>
+      <c r="T75" s="6" t="n"/>
+      <c r="U75" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:U65"/>
+  <autoFilter ref="A5:U75"/>
   <mergeCells count="1">
     <mergeCell ref="A2:V2"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="D6:D65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D6:D75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Obbligo di legge,Incentivi / fondi,Annunci di lavoro,Recensioni negative,Acquisizioni di verticali,Forum / community,Altro"</formula1>
     </dataValidation>
-    <dataValidation sqref="T6:T65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="T6:T75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da studiare,In studio,Da intervistare,Intervistata,Scartata,Scelta"</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:R65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="K6:R75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
@@ -3162,4 +4165,308 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fonti dei segnali (consultate il 03/11/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Quasi tutte sono stampa di settore e blog di consulenza, non testi ufficiali: le date vanno confermate sulla fonte primaria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>NIS2</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>https://www.noze.it/insights/nis2-pmi-cyberagent/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>https://www.agendadigitale.eu/sicurezza/nis2-scadenze-2026-la-guida-per-le-piccole-imprese/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>AI Act</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>https://www.agendadigitale.eu/industry-4-0/digital-omnibus-e-ai-act-cosa-puo-slittare-e-cosa-va-fatto-prima-di-agosto-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>https://www.noze.it/insights/ai-act-digital-omnibus-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Cyber Resilience Act</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>https://www.agendadigitale.eu/sicurezza/cyber-resilience-act-la-scadenza-chiave-arriva-l11-settembre-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>https://www.ipsoa.it/documents/quotidiano/2026/09/02/cyber-resilience-act-11-settembre-2026-scatta-obbligo-segnalare-vulnerabilita-incidenti-gravi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Direttiva RED</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>https://www.tuvsud.com/en-us/services/product-certification/red-cybersecurity-requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yarix.com/Advisory-and-Consulting-Services/RED-Compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Regolamento Macchine</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>https://certifico.com/macchine/regolamento-ue-2023-1230</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>https://www.ilsussidiario.net/news/regolamento-macchine-ue-rosa-ucimu-mancano-criteri-comuni-e-chiari-serve-una-proroga/2986256/amp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Trasparenza retributiva</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>https://quifinanza.it/lavoro/trasparenza-salariale-7-giugno-2026/960990/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>https://www.partitaiva.it/trasparenza-salariale/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>PPWR</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>https://www.assolombarda.it/servizi/ambiente/informazioni/ppwr-dal-12-agosto-in-applicazione-il-nuovo-regolamento-ue-sugli-imballaggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Passaporto digitale di prodotto</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>https://www.bluestonepim.com/blog/digital-product-passport-for-batteries</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>https://www.pmi.it/tecnologia/prodotti-e-servizi-ict/492107/passaporto-digitale-prodotto.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Accessibilità (EAA)</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>https://www.agendadigitale.eu/mercati-digitali/ecommerce/siti-ecommerce-accessibili-guida-in-5-step-per-evitare-sanzioni/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>https://www.iubenda.com/it/help/178476-accessibilita-101/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Iperammortamento 2026</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>https://www.agendadigitale.eu/industry-4-0/iperammortamento-2026-la-guida-cose-e-come-fare-le-comunicazioni-al-gse/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>https://pasqualepillitteri.it/perizia-iperammortamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Acquisizioni TeamSystem / Zucchetti</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>https://aventis-advisors.com/teamsystem-acquisitions/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Piano Italia 1 Giga</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>https://www.editorialedomani.it/economia/banda-ultralarga-cantieri-obiettivi-pnrr-ritardi-regioni-oqbs3i02</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>https://tariffe.segugio.it/news-tariffe/italia-1-giga-nuovi-ritardi-per-la-banda-ultra-larga-cosa-sta-succedendo-00043657.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>FWA e frequenze 26 GHz</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>https://tariffe.segugio.it/news-tariffe/internet-senza-fibra-la-fwa-supera-2-7-milioni-di-linee-00047779.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>https://www.smartworld.it/news/frequenze-5g-26-ghz-gara-italia-agosto-2026.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Comunità energetiche (CER)</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="inlineStr">
+        <is>
+          <t>https://www.infobuildenergia.it/approfondimenti/cer-comunita-energetiche-in-italia/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId25"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
freelance: Fase 2, stime di mercato per le 9 nicchie selezionate e quota necessaria per 1 M€
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNxVApXF9MzdDwSEC8TCy4
</commit_message>
<xml_diff>
--- a/freelance/griglia-nicchie.xlsx
+++ b/freelance/griglia-nicchie.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteri" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista lunga" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$U$75</definedName>
@@ -21,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <name val="Calibri"/>
@@ -109,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,14 +141,24 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -953,9 +966,17 @@
           <t>Noze; Agenda Digitale</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="F6" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Stampa di settore: 20.000–50.000 enti potenzialmente coinvolti (non registrati) (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>1500</v>
+      </c>
       <c r="I6" s="11">
         <f>IF(H6&gt;0,ROUND(1000000/H6,0),"")</f>
         <v/>
@@ -1008,9 +1029,17 @@
           <t>Noze; Agenda Digitale</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="F7" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mia ipotesi: numero di MSP e studi di consulenza IT rilevanti (nessun dato trovato) (affidabilità: Bassa)</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>2400</v>
+      </c>
       <c r="I7" s="11">
         <f>IF(H7&gt;0,ROUND(1000000/H7,0),"")</f>
         <v/>
@@ -1063,9 +1092,17 @@
           <t>Agenda Digitale; IPSOA</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="F8" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>ANIE: ~1.100 aziende associate (altre fonti: 1.600); più costruttori con software. Perimetro CRA non trovato (affidabilità: Bassa)</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>3000</v>
+      </c>
       <c r="I8" s="11">
         <f>IF(H8&gt;0,ROUND(1000000/H8,0),"")</f>
         <v/>
@@ -1118,9 +1155,17 @@
           <t>TÜV SÜD; Yarix</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="10" t="n"/>
+      <c r="F9" s="10" t="n">
+        <v>800</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Mia ipotesi: produttori e importatori di apparecchi radio in Italia (nessun dato trovato) (affidabilità: Bassa)</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>4000</v>
+      </c>
       <c r="I9" s="11">
         <f>IF(H9&gt;0,ROUND(1000000/H9,0),"")</f>
         <v/>
@@ -1173,9 +1218,17 @@
           <t>Certifico; UCIMU</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="F10" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Federmacchine 2020: 5.050 imprese (dato vecchio) (affidabilità: Media-bassa)</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>2500</v>
+      </c>
       <c r="I10" s="11">
         <f>IF(H10&gt;0,ROUND(1000000/H10,0),"")</f>
         <v/>
@@ -1503,9 +1556,17 @@
           <t>Agenda Digitale; Pasquale Pillitteri</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="10" t="n"/>
+      <c r="F16" s="10" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>CNI 2020: 4,5%–9% degli ingegneri ha firmato perizie, in media 10 ciascuno (+ ordine di grandezza mio) (affidabilità: Bassa)</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>600</v>
+      </c>
       <c r="I16" s="11">
         <f>IF(H16&gt;0,ROUND(1000000/H16,0),"")</f>
         <v/>
@@ -1558,9 +1619,17 @@
           <t>Domani</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="10" t="n"/>
+      <c r="F17" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Mia ipotesi: nessun dato trovato sul numero di imprese di posa (affidabilità: Bassa)</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>2000</v>
+      </c>
       <c r="I17" s="11">
         <f>IF(H17&gt;0,ROUND(1000000/H17,0),"")</f>
         <v/>
@@ -1723,9 +1792,17 @@
           <t>Segugio (dati AGCOM)</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="10" t="n"/>
+      <c r="F20" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Consulente 2022: 'centinaia' di WISP in Italia (affidabilità: Bassa)</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>1500</v>
+      </c>
       <c r="I20" s="11">
         <f>IF(H20&gt;0,ROUND(1000000/H20,0),"")</f>
         <v/>
@@ -1998,9 +2075,17 @@
           <t>idea precedente</t>
         </is>
       </c>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="10" t="n"/>
+      <c r="F25" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Accredia (31/12/2025): 1.448 laboratori di prova e 228 di taratura/altro; più laboratori interni non contati (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>1200</v>
+      </c>
       <c r="I25" s="11">
         <f>IF(H25&gt;0,ROUND(1000000/H25,0),"")</f>
         <v/>
@@ -3870,6 +3955,712 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fase 2 — dimensione dei mercati e quota necessaria per 1 M€ di ricavi (solo Italia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Numero di aziende: da fonti dove esistono, altrimenti ipotesi mie, con affidabilità indicata. I PREZZI SONO IPOTESI da validare nelle interviste. Le celle in blu si possono cambiare. 'Quota necessaria' = clienti per 1 M€ diviso aziende target: sopra circa il 10% il mercato italiano è troppo piccolo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Margine operativo ipotizzato</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Tassazione combinata (società + dividendi)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>0.465</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Obiettivo netto mensile (€)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Netto mensile con 1 M€ di ricavi (€)</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>ROUND(1000000*B4*(1-B5)/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Ricavi annui necessari per l'obiettivo (€)</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>ROUND(B6*12/(B4*(1-B5)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Nicchia</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Aziende target (bassa)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Aziende target (base)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Aziende target (alta)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Fonte della stima</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Affidabilità</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Prezzo annuo (bassa) €</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Prezzo annuo (base) €</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Prezzo annuo (alta) €</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Clienti per 1 M€ (base)</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Quota necessaria (base)</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Quota (caso favorevole)</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Quota (caso sfavorevole)</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Lettura</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>NIS2 per PMI</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Stampa di settore: 20.000–50.000 enti potenzialmente coinvolti (non registrati)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J11" s="11">
+        <f>ROUND(1000000/H11,0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="16">
+        <f>J11/C11</f>
+        <v/>
+      </c>
+      <c r="L11" s="17">
+        <f>(1000000/I11)/D11</f>
+        <v/>
+      </c>
+      <c r="M11" s="17">
+        <f>(1000000/G11)/B11</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Base ampia, ma mercato affollato di consulenti: serve un canale forte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>NIS2 per MSP e consulenti</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Mia ipotesi: numero di MSP e studi di consulenza IT rilevanti (nessun dato trovato)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J12" s="11">
+        <f>ROUND(1000000/H12,0)</f>
+        <v/>
+      </c>
+      <c r="K12" s="16">
+        <f>J12/C12</f>
+        <v/>
+      </c>
+      <c r="L12" s="17">
+        <f>(1000000/I12)/D12</f>
+        <v/>
+      </c>
+      <c r="M12" s="17">
+        <f>(1000000/G12)/B12</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Vendi al canale: meno clienti ma con più aziende ciascuno. Da confrontare con le piattaforme esistenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Cyber Resilience Act</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>ANIE: ~1.100 aziende associate (altre fonti: 1.600); più costruttori con software. Perimetro CRA non trovato</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J13" s="11">
+        <f>ROUND(1000000/H13,0)</f>
+        <v/>
+      </c>
+      <c r="K13" s="16">
+        <f>J13/C13</f>
+        <v/>
+      </c>
+      <c r="L13" s="17">
+        <f>(1000000/I13)/D13</f>
+        <v/>
+      </c>
+      <c r="M13" s="17">
+        <f>(1000000/G13)/B13</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Norma europea: il mercato vero è più grande dell'Italia, ma va servito in inglese e con concorrenti internazionali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Direttiva RED (radio/IoT)</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>800</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Mia ipotesi: produttori e importatori di apparecchi radio in Italia (nessun dato trovato)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J14" s="11">
+        <f>ROUND(1000000/H14,0)</f>
+        <v/>
+      </c>
+      <c r="K14" s="16">
+        <f>J14/C14</f>
+        <v/>
+      </c>
+      <c r="L14" s="17">
+        <f>(1000000/I14)/D14</f>
+        <v/>
+      </c>
+      <c r="M14" s="17">
+        <f>(1000000/G14)/B14</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Troppo piccolo come solo mercato italiano; ha senso solo come prodotto europeo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Regolamento Macchine</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Federmacchine 2020: 5.050 imprese (dato vecchio)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Media-bassa</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J15" s="11">
+        <f>ROUND(1000000/H15,0)</f>
+        <v/>
+      </c>
+      <c r="K15" s="16">
+        <f>J15/C15</f>
+        <v/>
+      </c>
+      <c r="L15" s="17">
+        <f>(1000000/I15)/D15</f>
+        <v/>
+      </c>
+      <c r="M15" s="17">
+        <f>(1000000/G15)/B15</f>
+        <v/>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Mercato ben definito e vicino a te; la scadenza (20/01/2027) può slittare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Iperammortamento 2026 (perizie)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>CNI 2020: 4,5%–9% degli ingegneri ha firmato perizie, in media 10 ciascuno (+ ordine di grandezza mio)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J16" s="11">
+        <f>ROUND(1000000/H16,0)</f>
+        <v/>
+      </c>
+      <c r="K16" s="16">
+        <f>J16/C16</f>
+        <v/>
+      </c>
+      <c r="L16" s="17">
+        <f>(1000000/I16)/D16</f>
+        <v/>
+      </c>
+      <c r="M16" s="17">
+        <f>(1000000/G16)/B16</f>
+        <v/>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Tanti utenti ma prezzo basso: serve come aggiunta a un prodotto più grande.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Fibra ottica (posa)</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Mia ipotesi: nessun dato trovato sul numero di imprese di posa</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J17" s="11">
+        <f>ROUND(1000000/H17,0)</f>
+        <v/>
+      </c>
+      <c r="K17" s="16">
+        <f>J17/C17</f>
+        <v/>
+      </c>
+      <c r="L17" s="17">
+        <f>(1000000/I17)/D17</f>
+        <v/>
+      </c>
+      <c r="M17" s="17">
+        <f>(1000000/G17)/B17</f>
+        <v/>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Mercato piccolo e dipendente da pochi committenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>FWA (piccoli operatori)</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Consulente 2022: 'centinaia' di WISP in Italia</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>800</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J18" s="11">
+        <f>ROUND(1000000/H18,0)</f>
+        <v/>
+      </c>
+      <c r="K18" s="16">
+        <f>J18/C18</f>
+        <v/>
+      </c>
+      <c r="L18" s="17">
+        <f>(1000000/I18)/D18</f>
+        <v/>
+      </c>
+      <c r="M18" s="17">
+        <f>(1000000/G18)/B18</f>
+        <v/>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Troppo piccolo come mercato solo italiano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Report di collaudo</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Accredia (31/12/2025): 1.448 laboratori di prova e 228 di taratura/altro; più laboratori interni non contati</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J19" s="11">
+        <f>ROUND(1000000/H19,0)</f>
+        <v/>
+      </c>
+      <c r="K19" s="16">
+        <f>J19/C19</f>
+        <v/>
+      </c>
+      <c r="L19" s="17">
+        <f>(1000000/I19)/D19</f>
+        <v/>
+      </c>
+      <c r="M19" s="17">
+        <f>(1000000/G19)/B19</f>
+        <v/>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Mercato di nicchia; gli strumenti di misura hanno già report inclusi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Come leggerla</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Le norme europee (CRA, RED, Macchine) si applicano in tutta l'UE: il mercato reale può essere molte volte quello italiano, ma richiede un prodotto in inglese e concorrenti internazionali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Per numeri precisi sulle aziende per codice ATECO e classe di addetti servono le tavole Istat (ASIA) su IstatData: scaricale e le analizzo. Dal mio ambiente non sono raggiungibili.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Nessun numero di questo foglio è un dato di mercato verificato per il tuo prodotto: sono ordini di grandezza per scartare le nicchie troppo piccole.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A23:N23"/>
+    <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A22:N22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3895,238 +4686,238 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Segmento</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Quota stimata</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Aziende (stima)</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Verificato?</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>Fonte verificata</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Manifattura avanzata e meccanica</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>26–28%</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>11.000–11.500</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E5" s="16" t="n"/>
+      <c r="E5" s="23" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Commercio all'ingrosso B2B</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>20–22%</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>8.500–9.000</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E6" s="16" t="n"/>
+      <c r="E6" s="23" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Servizi corporate, ICT e software</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>12–14%</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>5.000–5.800</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E7" s="16" t="n"/>
+      <c r="E7" s="23" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Costruzioni, impiantistica, real estate B2B</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>10–12%</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>4.200–4.800</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E8" s="16" t="n"/>
+      <c r="E8" s="23" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Chimica, polimeri, gomma-plastica</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>7–8%</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>3.000–3.300</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E9" s="16" t="n"/>
+      <c r="E9" s="23" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Logistica, spedizioni e trasporti B2B</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>6–7%</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>2.500–2.900</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E10" s="16" t="n"/>
+      <c r="E10" s="23" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Farmaceutica, biotech, dispositivi medici</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>4–5%</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>1.600–2.000</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E11" s="16" t="n"/>
+      <c r="E11" s="23" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Energia, ambiente, utilities B2B</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>3–4%</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>1.300–1.600</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E12" s="16" t="n"/>
+      <c r="E12" s="23" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Telecomunicazioni e reti</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>1,5–2%</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>600–800</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E13" s="16" t="n"/>
+      <c r="E13" s="23" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -4136,21 +4927,21 @@
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Quota di aziende lombarde con ricavi &gt;1 M€ per forma giuridica: ditte individuali &lt;0,5%, società di persone ~17%, società di capitali ~34% (fornite da te, senza fonte).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>B2B contro B2C: ~11-12% delle imprese B2B sopra 1 M€ contro ~2% delle B2C (altro chatbot, senza fonte). La direzione è plausibile, il rapporto 5-6x no.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Ripartizione B2B/B2C per forma giuridica: individuali 65/35, persone 55/45, capitali 60/40 (tue stime).</t>
         </is>
@@ -4167,13 +4958,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4183,12 +4974,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fonti dei segnali (consultate il 03/11/2026)</t>
+          <t>Fonti dei segnali (consultate fino al 30/10/2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Quasi tutte sono stampa di settore e blog di consulenza, non testi ufficiali: le date vanno confermate sulla fonte primaria.</t>
         </is>
@@ -4200,14 +4991,14 @@
           <t>NIS2</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>https://www.noze.it/insights/nis2-pmi-cyberagent/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/sicurezza/nis2-scadenze-2026-la-guida-per-le-piccole-imprese/</t>
         </is>
@@ -4219,14 +5010,14 @@
           <t>AI Act</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/industry-4-0/digital-omnibus-e-ai-act-cosa-puo-slittare-e-cosa-va-fatto-prima-di-agosto-2026/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>https://www.noze.it/insights/ai-act-digital-omnibus-2026/</t>
         </is>
@@ -4238,14 +5029,14 @@
           <t>Cyber Resilience Act</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/sicurezza/cyber-resilience-act-la-scadenza-chiave-arriva-l11-settembre-2026/</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>https://www.ipsoa.it/documents/quotidiano/2026/09/02/cyber-resilience-act-11-settembre-2026-scatta-obbligo-segnalare-vulnerabilita-incidenti-gravi</t>
         </is>
@@ -4257,14 +5048,14 @@
           <t>Direttiva RED</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>https://www.tuvsud.com/en-us/services/product-certification/red-cybersecurity-requirements</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>https://www.yarix.com/Advisory-and-Consulting-Services/RED-Compliance</t>
         </is>
@@ -4276,14 +5067,14 @@
           <t>Regolamento Macchine</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>https://certifico.com/macchine/regolamento-ue-2023-1230</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>https://www.ilsussidiario.net/news/regolamento-macchine-ue-rosa-ucimu-mancano-criteri-comuni-e-chiari-serve-una-proroga/2986256/amp/</t>
         </is>
@@ -4295,14 +5086,14 @@
           <t>Trasparenza retributiva</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>https://quifinanza.it/lavoro/trasparenza-salariale-7-giugno-2026/960990/</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B20" s="25" t="inlineStr">
         <is>
           <t>https://www.partitaiva.it/trasparenza-salariale/</t>
         </is>
@@ -4314,7 +5105,7 @@
           <t>PPWR</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>https://www.assolombarda.it/servizi/ambiente/informazioni/ppwr-dal-12-agosto-in-applicazione-il-nuovo-regolamento-ue-sugli-imballaggi</t>
         </is>
@@ -4326,14 +5117,14 @@
           <t>Passaporto digitale di prodotto</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>https://www.bluestonepim.com/blog/digital-product-passport-for-batteries</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="19" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>https://www.pmi.it/tecnologia/prodotti-e-servizi-ict/492107/passaporto-digitale-prodotto.html</t>
         </is>
@@ -4345,14 +5136,14 @@
           <t>Accessibilità (EAA)</t>
         </is>
       </c>
-      <c r="B27" s="19" t="inlineStr">
+      <c r="B27" s="25" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/mercati-digitali/ecommerce/siti-ecommerce-accessibili-guida-in-5-step-per-evitare-sanzioni/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="19" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>https://www.iubenda.com/it/help/178476-accessibilita-101/</t>
         </is>
@@ -4364,14 +5155,14 @@
           <t>Iperammortamento 2026</t>
         </is>
       </c>
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/industry-4-0/iperammortamento-2026-la-guida-cose-e-come-fare-le-comunicazioni-al-gse/</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="19" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>https://pasqualepillitteri.it/perizia-iperammortamento</t>
         </is>
@@ -4383,7 +5174,7 @@
           <t>Acquisizioni TeamSystem / Zucchetti</t>
         </is>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>https://aventis-advisors.com/teamsystem-acquisitions/</t>
         </is>
@@ -4395,14 +5186,14 @@
           <t>Piano Italia 1 Giga</t>
         </is>
       </c>
-      <c r="B35" s="19" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>https://www.editorialedomani.it/economia/banda-ultralarga-cantieri-obiettivi-pnrr-ritardi-regioni-oqbs3i02</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>https://tariffe.segugio.it/news-tariffe/italia-1-giga-nuovi-ritardi-per-la-banda-ultra-larga-cosa-sta-succedendo-00043657.aspx</t>
         </is>
@@ -4414,14 +5205,14 @@
           <t>FWA e frequenze 26 GHz</t>
         </is>
       </c>
-      <c r="B38" s="19" t="inlineStr">
+      <c r="B38" s="25" t="inlineStr">
         <is>
           <t>https://tariffe.segugio.it/news-tariffe/internet-senza-fibra-la-fwa-supera-2-7-milioni-di-linee-00047779.aspx</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="19" t="inlineStr">
+      <c r="B39" s="25" t="inlineStr">
         <is>
           <t>https://www.smartworld.it/news/frequenze-5g-26-ghz-gara-italia-agosto-2026.html</t>
         </is>
@@ -4430,10 +5221,50 @@
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
+          <t>Fase 2 — numeri di mercato</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="inlineStr">
+        <is>
+          <t>https://accredia.it/wp-content/uploads/2024/07/Cartella-stampa-breve-dati-al-31-12-2025_ITA-1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="25" t="inlineStr">
+        <is>
+          <t>https://assomac.it/media/documents/rapporto_federmacchine_2020.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>https://anie.it/federazione/chi-siamo/rapporto-annuale-2025_def</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="25" t="inlineStr">
+        <is>
+          <t>https://www.cni.it/images/eventi/2021/01_Lelaborazione_delle_perizie_13lug2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="25" t="inlineStr">
+        <is>
+          <t>https://www.fibertelecom.com/wt/2022/PDF/02-puglia/FTWWT2022-puglia-03.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
           <t>Comunità energetiche (CER)</t>
         </is>
       </c>
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B47" s="25" t="inlineStr">
         <is>
           <t>https://www.infobuildenergia.it/approfondimenti/cer-comunita-energetiche-in-italia/</t>
         </is>
@@ -4466,6 +5297,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
freelance: sostituisce le ipotesi con i dati Istat 2024 (unità locali per ATECO e classe di addetti) e aggiunge il file sorgente
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNxVApXF9MzdDwSEC8TCy4
</commit_message>
<xml_diff>
--- a/freelance/griglia-nicchie.xlsx
+++ b/freelance/griglia-nicchie.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteri" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista lunga" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istat 2024" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$U$75</definedName>
@@ -112,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -154,8 +155,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -967,11 +969,11 @@
         </is>
       </c>
       <c r="F6" s="10" t="n">
-        <v>20000</v>
+        <v>13500</v>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Stampa di settore: 20.000–50.000 enti potenzialmente coinvolti (non registrati) (affidabilità: Media)</t>
+          <t>Istat ASIA 2024: 13.574 unità locali con 50+ addetti nei settori NIS2 (perimetro mio, approssimato). Stampa: 20.000-50.000 enti. Sono unità locali: limite superiore (affidabilità: Media)</t>
         </is>
       </c>
       <c r="H6" s="10" t="n">
@@ -1030,11 +1032,11 @@
         </is>
       </c>
       <c r="F7" s="10" t="n">
-        <v>5000</v>
+        <v>4400</v>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Mia ipotesi: numero di MSP e studi di consulenza IT rilevanti (nessun dato trovato) (affidabilità: Bassa)</t>
+          <t>Istat 2024: ATECO 62.02/62.03/62.09 e 63.11 con 10+ addetti (unità locali); alto = tutto 62 e 63.1 con 10+ (affidabilità: Media)</t>
         </is>
       </c>
       <c r="H7" s="10" t="n">
@@ -1093,11 +1095,11 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>3000</v>
+        <v>4400</v>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>ANIE: ~1.100 aziende associate (altre fonti: 1.600); più costruttori con software. Perimetro CRA non trovato (affidabilità: Bassa)</t>
+          <t>Istat 2024: ATECO 26 (1.692), 26+27 (4.396), + 28 e software 62.01 con 10+ (17.011); solo una parte produce prodotti con elementi digitali (affidabilità: Media-bassa)</t>
         </is>
       </c>
       <c r="H8" s="10" t="n">
@@ -1156,11 +1158,11 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>800</v>
+        <v>780</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Mia ipotesi: produttori e importatori di apparecchi radio in Italia (nessun dato trovato) (affidabilità: Bassa)</t>
+          <t>Istat 2024: ATECO 26.3 (781 unità locali, 254 con 10+); alto = ATECO 26 con 10+ (1.692). Gli importatori non sono inclusi (affidabilità: Media-bassa)</t>
         </is>
       </c>
       <c r="H9" s="10" t="n">
@@ -1219,11 +1221,11 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Federmacchine 2020: 5.050 imprese (dato vecchio) (affidabilità: Media-bassa)</t>
+          <t>Istat 2024: ATECO 28 = 22.720 unità locali, 9.059 con 10+, 2.179 con 50+. Controllo: Federmacchine 2020, 5.050 imprese associate (affidabilità: Media)</t>
         </is>
       </c>
       <c r="H10" s="10" t="n">
@@ -1561,7 +1563,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>CNI 2020: 4,5%–9% degli ingegneri ha firmato perizie, in media 10 ciascuno (+ ordine di grandezza mio) (affidabilità: Bassa)</t>
+          <t>CNI 2020: 4,5%-9% degli ingegneri ha firmato perizie, in media 10 ciascuno (+ ordine di grandezza mio) (affidabilità: Bassa)</t>
         </is>
       </c>
       <c r="H16" s="10" t="n">
@@ -1620,11 +1622,11 @@
         </is>
       </c>
       <c r="F17" s="10" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Mia ipotesi: nessun dato trovato sul numero di imprese di posa (affidabilità: Bassa)</t>
+          <t>Istat 2024: ATECO 42.22 = 805 unità locali (401 con 10+); alto = + 43.21 con 10+ (5.781). La posa è distribuita su più codici (affidabilità: Media-bassa)</t>
         </is>
       </c>
       <c r="H17" s="10" t="n">
@@ -1793,11 +1795,11 @@
         </is>
       </c>
       <c r="F20" s="10" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Consulente 2022: 'centinaia' di WISP in Italia (affidabilità: Bassa)</t>
+          <t>Istat 2024: ATECO 61.10 = 1.315 e 61.20 = 226 unità locali. I WISP non sono isolabili; base = mio giudizio (affidabilità: Bassa)</t>
         </is>
       </c>
       <c r="H20" s="10" t="n">
@@ -2076,11 +2078,11 @@
         </is>
       </c>
       <c r="F25" s="10" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Accredia (31/12/2025): 1.448 laboratori di prova e 228 di taratura/altro; più laboratori interni non contati (affidabilità: Media)</t>
+          <t>Istat 2024: ATECO 71.20 = 9.362 unità locali, 1.041 con 10+; 71.20.1 prodotti = 3.867. Accredia: 1.448 laboratori di prova (affidabilità: Media)</t>
         </is>
       </c>
       <c r="H25" s="10" t="n">
@@ -4119,17 +4121,17 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>10000</v>
+        <v>7000</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>20000</v>
+        <v>13500</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Stampa di settore: 20.000–50.000 enti potenzialmente coinvolti (non registrati)</t>
+          <t>Istat ASIA 2024: 13.574 unità locali con 50+ addetti nei settori NIS2 (perimetro mio, approssimato). Stampa: 20.000-50.000 enti. Sono unità locali: limite superiore</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -4175,22 +4177,22 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2000</v>
+        <v>2700</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>5000</v>
+        <v>4400</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Mia ipotesi: numero di MSP e studi di consulenza IT rilevanti (nessun dato trovato)</t>
+          <t>Istat 2024: ATECO 62.02/62.03/62.09 e 63.11 con 10+ addetti (unità locali); alto = tutto 62 e 63.1 con 10+</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
@@ -4231,22 +4233,22 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>1100</v>
+        <v>1700</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>3000</v>
+        <v>4400</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>8000</v>
+        <v>17000</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>ANIE: ~1.100 aziende associate (altre fonti: 1.600); più costruttori con software. Perimetro CRA non trovato</t>
+          <t>Istat 2024: ATECO 26 (1.692), 26+27 (4.396), + 28 e software 62.01 con 10+ (17.011); solo una parte produce prodotti con elementi digitali</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Media-bassa</t>
         </is>
       </c>
       <c r="G13" s="10" t="n">
@@ -4287,22 +4289,22 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>800</v>
+        <v>780</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>2000</v>
+        <v>1700</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Mia ipotesi: produttori e importatori di apparecchi radio in Italia (nessun dato trovato)</t>
+          <t>Istat 2024: ATECO 26.3 (781 unità locali, 254 con 10+); alto = ATECO 26 con 10+ (1.692). Gli importatori non sono inclusi</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Media-bassa</t>
         </is>
       </c>
       <c r="G14" s="10" t="n">
@@ -4343,22 +4345,22 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>3000</v>
+        <v>2200</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>8000</v>
+        <v>22700</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Federmacchine 2020: 5.050 imprese (dato vecchio)</t>
+          <t>Istat 2024: ATECO 28 = 22.720 unità locali, 9.059 con 10+, 2.179 con 50+. Controllo: Federmacchine 2020, 5.050 imprese associate</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Media-bassa</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G15" s="10" t="n">
@@ -4409,7 +4411,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>CNI 2020: 4,5%–9% degli ingegneri ha firmato perizie, in media 10 ciascuno (+ ordine di grandezza mio)</t>
+          <t>CNI 2020: 4,5%-9% degli ingegneri ha firmato perizie, in media 10 ciascuno (+ ordine di grandezza mio)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -4455,22 +4457,22 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>3000</v>
+        <v>6600</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Mia ipotesi: nessun dato trovato sul numero di imprese di posa</t>
+          <t>Istat 2024: ATECO 42.22 = 805 unità locali (401 con 10+); alto = + 43.21 con 10+ (5.781). La posa è distribuita su più codici</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Media-bassa</t>
         </is>
       </c>
       <c r="G17" s="10" t="n">
@@ -4511,17 +4513,17 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>1000</v>
+        <v>1300</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Consulente 2022: 'centinaia' di WISP in Italia</t>
+          <t>Istat 2024: ATECO 61.10 = 1.315 e 61.20 = 226 unità locali. I WISP non sono isolabili; base = mio giudizio</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -4567,17 +4569,17 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>1700</v>
+        <v>1000</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>10000</v>
+        <v>3900</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Accredia (31/12/2025): 1.448 laboratori di prova e 228 di taratura/altro; più laboratori interni non contati</t>
+          <t>Istat 2024: ATECO 71.20 = 9.362 unità locali, 1.041 con 10+; 71.20.1 prodotti = 3.867. Accredia: 1.448 laboratori di prova</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -4626,14 +4628,14 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>Le norme europee (CRA, RED, Macchine) si applicano in tutta l'UE: il mercato reale può essere molte volte quello italiano, ma richiede un prodotto in inglese e concorrenti internazionali.</t>
+          <t>Il numero di aziende viene da Istat 2024 (unità locali, quindi limiti superiori) dove è indicato; le ipotesi residue sono segnate nella colonna Affidabilità. Le norme europee (CRA, RED, Macchine) si applicano in tutta l'UE: il mercato reale può essere molte volte quello italiano, ma richiede un prodotto in inglese e concorrenti internazionali.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>Per numeri precisi sulle aziende per codice ATECO e classe di addetti servono le tavole Istat (ASIA) su IstatData: scaricale e le analizzo. Dal mio ambiente non sono raggiungibili.</t>
+          <t>Prossimo passo di precisione: il perimetro NIS2 e le quote di prodotti con elementi digitali sono mie approssimazioni, da affinare nelle interviste.</t>
         </is>
       </c>
     </row>
@@ -4661,6 +4663,1037 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Istat ASIA 2024 — unità locali delle imprese attive per classe di addetti (estratto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: Istat, 'Classe di addetti, settori economici (Ateco 5 cifre) - Italia', anno 2024. ATTENZIONE: sono UNITÀ LOCALI, non imprese: una società con più sedi conta più volte, quindi sono limiti superiori. File completo in freelance/dati/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Codice</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Attività</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>UL 0-9</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>UL 10-49</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>UL 50-249</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>UL 250+</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>UL totale</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>UL con 10+</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>UL con 50+</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Addetti totali (medi annui)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di computer e prodotti di elettronica e ottica, apparecchi elettromedicali, apparecchi di misurazione e di orologi</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>4306</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>1282</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>371</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>39</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>5998</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>1692</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>410</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <v>104511.99</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>263</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di apparecchiature per le telecomunicazioni</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>527</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>189</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>56</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>781</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>254</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>65</v>
+      </c>
+      <c r="J6" s="20" t="n">
+        <v>17059.01</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>265</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di strumenti e apparecchi di misurazione, prova e navigazione, orologi</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>755</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>288</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>109</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>1158</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>403</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>115</v>
+      </c>
+      <c r="J7" s="20" t="n">
+        <v>21838.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di apparecchiature elettriche ed apparecchiature per uso domestico non elettriche</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>6161</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>2119</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>521</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>64</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>8865</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>2704</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>585</v>
+      </c>
+      <c r="J8" s="20" t="n">
+        <v>147905.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>271</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di motori, generatori e trasformatori elettrici e di apparecchiature per la distribuzione e il controllo dell'elettricità</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>1611</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>701</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>185</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>2525</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>914</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>213</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>52232.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>273</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di cablaggi e apparecchiature di cablaggio</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>681</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>242</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>99</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>1026</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>345</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>103</v>
+      </c>
+      <c r="J10" s="20" t="n">
+        <v>19036.78</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>279</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di altre apparecchiature elettriche</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>2312</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>758</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>122</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>3197</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>885</v>
+      </c>
+      <c r="I11" s="20" t="n">
+        <v>127</v>
+      </c>
+      <c r="J11" s="20" t="n">
+        <v>34743.28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di macchinari ed apparecchiature nca</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>13661</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>6880</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>1967</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>212</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>22720</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>9059</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <v>2179</v>
+      </c>
+      <c r="J12" s="20" t="n">
+        <v>489551.23</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>281</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di macchine di impiego generale</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>1516</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>1016</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>440</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>68</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>3040</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>1524</v>
+      </c>
+      <c r="I13" s="20" t="n">
+        <v>508</v>
+      </c>
+      <c r="J13" s="20" t="n">
+        <v>105044.42</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>282</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di altre macchine di impiego generale</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>5470</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <v>2694</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>774</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>74</v>
+      </c>
+      <c r="G14" s="20" t="n">
+        <v>9012</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>3542</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <v>848</v>
+      </c>
+      <c r="J14" s="20" t="n">
+        <v>187206.72</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>283</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di macchine per l'agricoltura e la silvicoltura</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>962</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>464</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>108</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>1553</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>591</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <v>127</v>
+      </c>
+      <c r="J15" s="20" t="n">
+        <v>33472.05</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>284</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di macchine per la formatura dei metalli e di altre macchine utensili</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>1260</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>611</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>141</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="G16" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>767</v>
+      </c>
+      <c r="I16" s="20" t="n">
+        <v>156</v>
+      </c>
+      <c r="J16" s="20" t="n">
+        <v>39136.66</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>289</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Fabbricazione di altre macchine per impieghi speciali</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>4453</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>2095</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>504</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>36</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <v>7088</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>2635</v>
+      </c>
+      <c r="I17" s="20" t="n">
+        <v>540</v>
+      </c>
+      <c r="J17" s="20" t="n">
+        <v>124691.38</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>4222</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Costruzione di opere di pubblica utilità per l'energia elettrica e le telecomunicazioni</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="n">
+        <v>404</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>267</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>120</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="G18" s="20" t="n">
+        <v>805</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>401</v>
+      </c>
+      <c r="I18" s="20" t="n">
+        <v>134</v>
+      </c>
+      <c r="J18" s="20" t="n">
+        <v>24721.08</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>4321</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Installazione di impianti elettrici</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="n">
+        <v>67567</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <v>5339</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>431</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="G19" s="20" t="n">
+        <v>73348</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>5781</v>
+      </c>
+      <c r="I19" s="20" t="n">
+        <v>442</v>
+      </c>
+      <c r="J19" s="20" t="n">
+        <v>275831.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>6110</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Telecomunicazioni fisse</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="n">
+        <v>801</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>407</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>74</v>
+      </c>
+      <c r="F20" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="G20" s="20" t="n">
+        <v>1315</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <v>514</v>
+      </c>
+      <c r="I20" s="20" t="n">
+        <v>107</v>
+      </c>
+      <c r="J20" s="20" t="n">
+        <v>41897.35</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>6120</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Telecomunicazioni mobili</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="n">
+        <v>176</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="E21" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" s="20" t="n">
+        <v>226</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="J21" s="20" t="n">
+        <v>10233.93</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>6190</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Altre attività di telecomunicazione</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="n">
+        <v>3187</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>220</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <v>3426</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>239</v>
+      </c>
+      <c r="I22" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="J22" s="20" t="n">
+        <v>12419.78</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>6201</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Produzione di software non connesso all'edizione</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>21349</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>2886</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>573</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>97</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <v>24905</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <v>3556</v>
+      </c>
+      <c r="I23" s="20" t="n">
+        <v>670</v>
+      </c>
+      <c r="J23" s="20" t="n">
+        <v>205532.07</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>6202</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Consulenza nel settore delle tecnologie dell'informatica</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="n">
+        <v>30003</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>337</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="G24" s="20" t="n">
+        <v>31653</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <v>1650</v>
+      </c>
+      <c r="I24" s="20" t="n">
+        <v>375</v>
+      </c>
+      <c r="J24" s="20" t="n">
+        <v>122175.74</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>6203</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Gestione di strutture informatizzate</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>1008</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>119</v>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="20" t="n">
+        <v>1161</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <v>153</v>
+      </c>
+      <c r="I25" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="J25" s="20" t="n">
+        <v>7538.78</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>6209</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Altre attività dei servizi connessi alle tecnologie dell'informatica</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="n">
+        <v>11655</v>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>729</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>154</v>
+      </c>
+      <c r="F26" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="G26" s="20" t="n">
+        <v>12547</v>
+      </c>
+      <c r="H26" s="20" t="n">
+        <v>892</v>
+      </c>
+      <c r="I26" s="20" t="n">
+        <v>163</v>
+      </c>
+      <c r="J26" s="20" t="n">
+        <v>52353.85</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>6311</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Elaborazione dei dati, hosting e attività connesse</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>36015</v>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>1527</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>161</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>37717</v>
+      </c>
+      <c r="H27" s="20" t="n">
+        <v>1702</v>
+      </c>
+      <c r="I27" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="J27" s="20" t="n">
+        <v>115837.62</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>71201</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Collaudi e analisi tecniche di prodotti</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="n">
+        <v>3177</v>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>606</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>3867</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v>690</v>
+      </c>
+      <c r="I28" s="20" t="n">
+        <v>84</v>
+      </c>
+      <c r="J28" s="20" t="n">
+        <v>27828.3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>71202</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Controllo di qualità e certificazione di prodotti, processi e sistemi</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="n">
+        <v>5144</v>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>310</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="20" t="n">
+        <v>5495</v>
+      </c>
+      <c r="H29" s="20" t="n">
+        <v>351</v>
+      </c>
+      <c r="I29" s="20" t="n">
+        <v>41</v>
+      </c>
+      <c r="J29" s="20" t="n">
+        <v>19723.08</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>7112</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Attività degli studi d'ingegneria ed altri studi tecnici</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="n">
+        <v>154402</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>1097</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>197</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>155713</v>
+      </c>
+      <c r="H30" s="20" t="n">
+        <v>1311</v>
+      </c>
+      <c r="I30" s="20" t="n">
+        <v>214</v>
+      </c>
+      <c r="J30" s="20" t="n">
+        <v>227325.53</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:L2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4686,238 +5719,238 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Segmento</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Quota stimata</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Aziende (stima)</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Verificato?</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Fonte verificata</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Manifattura avanzata e meccanica</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>26–28%</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>11.000–11.500</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E5" s="23" t="n"/>
+      <c r="E5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Commercio all'ingrosso B2B</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>20–22%</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>8.500–9.000</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E6" s="23" t="n"/>
+      <c r="E6" s="24" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Servizi corporate, ICT e software</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>12–14%</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>5.000–5.800</t>
         </is>
       </c>
-      <c r="D7" s="22" t="inlineStr">
+      <c r="D7" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E7" s="23" t="n"/>
+      <c r="E7" s="24" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Costruzioni, impiantistica, real estate B2B</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>10–12%</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>4.200–4.800</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E8" s="23" t="n"/>
+      <c r="E8" s="24" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Chimica, polimeri, gomma-plastica</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>7–8%</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>3.000–3.300</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E9" s="23" t="n"/>
+      <c r="E9" s="24" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Logistica, spedizioni e trasporti B2B</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>6–7%</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>2.500–2.900</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E10" s="23" t="n"/>
+      <c r="E10" s="24" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Farmaceutica, biotech, dispositivi medici</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>4–5%</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>1.600–2.000</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr">
+      <c r="D11" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E11" s="23" t="n"/>
+      <c r="E11" s="24" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Energia, ambiente, utilities B2B</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>3–4%</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>1.300–1.600</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E12" s="23" t="n"/>
+      <c r="E12" s="24" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Telecomunicazioni e reti</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>1,5–2%</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>600–800</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E13" s="23" t="n"/>
+      <c r="E13" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -4958,13 +5991,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4979,7 +6012,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Quasi tutte sono stampa di settore e blog di consulenza, non testi ufficiali: le date vanno confermate sulla fonte primaria.</t>
         </is>
@@ -4991,14 +6024,14 @@
           <t>NIS2</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>https://www.noze.it/insights/nis2-pmi-cyberagent/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/sicurezza/nis2-scadenze-2026-la-guida-per-le-piccole-imprese/</t>
         </is>
@@ -5010,14 +6043,14 @@
           <t>AI Act</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/industry-4-0/digital-omnibus-e-ai-act-cosa-puo-slittare-e-cosa-va-fatto-prima-di-agosto-2026/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="25" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>https://www.noze.it/insights/ai-act-digital-omnibus-2026/</t>
         </is>
@@ -5029,14 +6062,14 @@
           <t>Cyber Resilience Act</t>
         </is>
       </c>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/sicurezza/cyber-resilience-act-la-scadenza-chiave-arriva-l11-settembre-2026/</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>https://www.ipsoa.it/documents/quotidiano/2026/09/02/cyber-resilience-act-11-settembre-2026-scatta-obbligo-segnalare-vulnerabilita-incidenti-gravi</t>
         </is>
@@ -5048,14 +6081,14 @@
           <t>Direttiva RED</t>
         </is>
       </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>https://www.tuvsud.com/en-us/services/product-certification/red-cybersecurity-requirements</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>https://www.yarix.com/Advisory-and-Consulting-Services/RED-Compliance</t>
         </is>
@@ -5067,14 +6100,14 @@
           <t>Regolamento Macchine</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>https://certifico.com/macchine/regolamento-ue-2023-1230</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="25" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>https://www.ilsussidiario.net/news/regolamento-macchine-ue-rosa-ucimu-mancano-criteri-comuni-e-chiari-serve-una-proroga/2986256/amp/</t>
         </is>
@@ -5086,14 +6119,14 @@
           <t>Trasparenza retributiva</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>https://quifinanza.it/lavoro/trasparenza-salariale-7-giugno-2026/960990/</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>https://www.partitaiva.it/trasparenza-salariale/</t>
         </is>
@@ -5105,7 +6138,7 @@
           <t>PPWR</t>
         </is>
       </c>
-      <c r="B22" s="25" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>https://www.assolombarda.it/servizi/ambiente/informazioni/ppwr-dal-12-agosto-in-applicazione-il-nuovo-regolamento-ue-sugli-imballaggi</t>
         </is>
@@ -5117,14 +6150,14 @@
           <t>Passaporto digitale di prodotto</t>
         </is>
       </c>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>https://www.bluestonepim.com/blog/digital-product-passport-for-batteries</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>https://www.pmi.it/tecnologia/prodotti-e-servizi-ict/492107/passaporto-digitale-prodotto.html</t>
         </is>
@@ -5136,14 +6169,14 @@
           <t>Accessibilità (EAA)</t>
         </is>
       </c>
-      <c r="B27" s="25" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/mercati-digitali/ecommerce/siti-ecommerce-accessibili-guida-in-5-step-per-evitare-sanzioni/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="25" t="inlineStr">
+      <c r="B28" s="26" t="inlineStr">
         <is>
           <t>https://www.iubenda.com/it/help/178476-accessibilita-101/</t>
         </is>
@@ -5155,14 +6188,14 @@
           <t>Iperammortamento 2026</t>
         </is>
       </c>
-      <c r="B30" s="25" t="inlineStr">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/industry-4-0/iperammortamento-2026-la-guida-cose-e-come-fare-le-comunicazioni-al-gse/</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="25" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>https://pasqualepillitteri.it/perizia-iperammortamento</t>
         </is>
@@ -5174,7 +6207,7 @@
           <t>Acquisizioni TeamSystem / Zucchetti</t>
         </is>
       </c>
-      <c r="B33" s="25" t="inlineStr">
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>https://aventis-advisors.com/teamsystem-acquisitions/</t>
         </is>
@@ -5186,14 +6219,14 @@
           <t>Piano Italia 1 Giga</t>
         </is>
       </c>
-      <c r="B35" s="25" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>https://www.editorialedomani.it/economia/banda-ultralarga-cantieri-obiettivi-pnrr-ritardi-regioni-oqbs3i02</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="25" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>https://tariffe.segugio.it/news-tariffe/italia-1-giga-nuovi-ritardi-per-la-banda-ultra-larga-cosa-sta-succedendo-00043657.aspx</t>
         </is>
@@ -5205,14 +6238,14 @@
           <t>FWA e frequenze 26 GHz</t>
         </is>
       </c>
-      <c r="B38" s="25" t="inlineStr">
+      <c r="B38" s="26" t="inlineStr">
         <is>
           <t>https://tariffe.segugio.it/news-tariffe/internet-senza-fibra-la-fwa-supera-2-7-milioni-di-linee-00047779.aspx</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="25" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>https://www.smartworld.it/news/frequenze-5g-26-ghz-gara-italia-agosto-2026.html</t>
         </is>
@@ -5224,47 +6257,54 @@
           <t>Fase 2 — numeri di mercato</t>
         </is>
       </c>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>https://esploradati.istat.it (dataset: Classe di addetti, settori economici (Ateco 5 cifre) - Italia, anno 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="26" t="inlineStr">
         <is>
           <t>https://accredia.it/wp-content/uploads/2024/07/Cartella-stampa-breve-dati-al-31-12-2025_ITA-1.pdf</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="25" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>https://assomac.it/media/documents/rapporto_federmacchine_2020.pdf</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="25" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="26" t="inlineStr">
         <is>
           <t>https://anie.it/federazione/chi-siamo/rapporto-annuale-2025_def</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="25" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="26" t="inlineStr">
         <is>
           <t>https://www.cni.it/images/eventi/2021/01_Lelaborazione_delle_perizie_13lug2021.pdf</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="25" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="26" t="inlineStr">
         <is>
           <t>https://www.fibertelecom.com/wt/2022/PDF/02-puglia/FTWWT2022-puglia-03.pdf</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>Comunità energetiche (CER)</t>
         </is>
       </c>
-      <c r="B47" s="25" t="inlineStr">
+      <c r="B48" s="26" t="inlineStr">
         <is>
           <t>https://www.infobuildenergia.it/approfondimenti/cer-comunita-energetiche-in-italia/</t>
         </is>
@@ -5301,7 +6341,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
freelance: aggiunge il criterio 'bisogno permanente', 5 nicchie evergreen e la durabilità nel foglio Fase 2
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNxVApXF9MzdDwSEC8TCy4
</commit_message>
<xml_diff>
--- a/freelance/griglia-nicchie.xlsx
+++ b/freelance/griglia-nicchie.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$U$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$V$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -596,12 +596,12 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Budget del cliente</t>
+          <t>Bisogno permanente</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>I clienti tipo hanno ricavi &gt;1 M€ e capacità di spesa?</t>
+          <t>Il bisogno esiste anche se non cambia nessuna legge e non c'è nessuna scadenza?</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
@@ -609,79 +609,79 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>1 = micro-imprese; 5 = PMI con &gt;1 M€ di ricavi e abitudine a pagare software</t>
+          <t>1 = nasce da una scadenza o da un'ondata normativa; 5 = problema operativo o di cassa che esiste sempre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Ricavi ricorrenti</t>
+          <t>Budget del cliente</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Il cliente paga ogni anno o ogni mese?</t>
+          <t>I clienti tipo hanno ricavi &gt;1 M€ e capacità di spesa?</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>1 = una tantum; 5 = abbonamento naturale</t>
+          <t>1 = micro-imprese; 5 = PMI con &gt;1 M€ di ricavi e abitudine a pagare software</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Scalabilità</t>
+          <t>Ricavi ricorrenti</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Quanto costa servire un cliente in più? Margine?</t>
+          <t>Il cliente paga ogni anno o ogni mese?</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>1 = molto lavoro per cliente; 5 = costo marginale quasi zero</t>
+          <t>1 = una tantum; 5 = abbonamento naturale</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Canale di vendita</t>
+          <t>Scalabilità</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Sai dove trovare i clienti e come raggiungerli?</t>
+          <t>Quanto costa servire un cliente in più? Margine?</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>1 = nessun canale chiaro; 5 = canale noto (associazioni, rivenditori, consulenti)</t>
+          <t>1 = molto lavoro per cliente; 5 = costo marginale quasi zero</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Concorrenza (5 = poca)</t>
+          <t>Canale di vendita</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Quanti concorrenti e quanto forti?</t>
+          <t>Sai dove trovare i clienti e come raggiungerli?</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -689,19 +689,19 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>1 = mercato saturo; 5 = pochi o nessuno ben posizionato</t>
+          <t>1 = nessun canale chiaro; 5 = canale noto (associazioni, rivenditori, consulenti)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Vantaggio tuo</t>
+          <t>Concorrenza (5 = poca)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Capisci il problema meglio di chi lo risolve oggi?</t>
+          <t>Quanti concorrenti e quanto forti?</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -709,38 +709,58 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>1 = nessun vantaggio; 5 = lo conosci dall'interno</t>
+          <t>1 = mercato saturo; 5 = pochi o nessuno ben posizionato</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>Vantaggio tuo</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Capisci il problema meglio di chi lo risolve oggi?</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>1 = nessun vantaggio; 5 = lo conosci dall'interno</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>Testabile a poco prezzo</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Puoi verificare la domanda con un prototipo e conversazioni, senza spendere?</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>1 = serve capitale; 5 = test in 2 settimane a costo zero</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Somma dei pesi</t>
         </is>
       </c>
-      <c r="C13" s="7">
-        <f>SUM(C5:C12)</f>
+      <c r="C14" s="7">
+        <f>SUM(C5:C13)</f>
         <v/>
       </c>
     </row>
@@ -779,9 +799,10 @@
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="40" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -836,6 +857,10 @@
         <f>Criteri!C12</f>
         <v/>
       </c>
+      <c r="S4" s="8">
+        <f>Criteri!C13</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -895,50 +920,55 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
+          <t>Bisogno permanente</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
           <t>Budget del cliente</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Ricavi ricorrenti</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Scalabilità</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Canale di vendita</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>Concorrenza (5 = poca)</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Vantaggio tuo</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>Testabile a poco prezzo</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>Punteggio ponderato (1-5)</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>Stato</t>
         </is>
       </c>
-      <c r="U5" s="3" t="inlineStr">
+      <c r="V5" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -992,16 +1022,17 @@
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="6" t="n"/>
       <c r="R6" s="6" t="n"/>
-      <c r="S6" s="4">
-        <f>IF(COUNT(K6:R6)=0,"",ROUND(SUMPRODUCT(K6:R6,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T6" s="6" t="inlineStr">
+      <c r="S6" s="6" t="n"/>
+      <c r="T6" s="4">
+        <f>IF(COUNT(K6:S6)=0,"",ROUND(SUMPRODUCT(K6:S6,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U6" s="6" t="inlineStr">
+      <c r="V6" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Notifica incidenti operativa dal 15/01/2026; misure di base con scadenze da ottobre 2026 per chi ha ricevuto la comunicazione ad aprile 2025. Mercato affollato di consulenti. Numero di imprese coinvolte non trovato.</t>
         </is>
@@ -1055,16 +1086,17 @@
       <c r="P7" s="6" t="n"/>
       <c r="Q7" s="6" t="n"/>
       <c r="R7" s="6" t="n"/>
-      <c r="S7" s="4">
-        <f>IF(COUNT(K7:R7)=0,"",ROUND(SUMPRODUCT(K7:R7,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T7" s="6" t="inlineStr">
+      <c r="S7" s="6" t="n"/>
+      <c r="T7" s="4">
+        <f>IF(COUNT(K7:S7)=0,"",ROUND(SUMPRODUCT(K7:S7,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U7" s="6" t="inlineStr">
+      <c r="V7" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Variante della precedente: vendi al canale, non alla PMI finale. Da confrontare con piattaforme esistenti.</t>
         </is>
@@ -1118,16 +1150,17 @@
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="6" t="n"/>
-      <c r="S8" s="4">
-        <f>IF(COUNT(K8:R8)=0,"",ROUND(SUMPRODUCT(K8:R8,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T8" s="6" t="inlineStr">
+      <c r="S8" s="6" t="n"/>
+      <c r="T8" s="4">
+        <f>IF(COUNT(K8:S8)=0,"",ROUND(SUMPRODUCT(K8:S8,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U8" s="6" t="inlineStr">
+      <c r="V8" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Obbligo di segnalazione dall'11/09/2026 (preallarme in 24 ore); piena applicazione 11/12/2027; sanzioni fino a 15 M€ (stampa). Vantaggio tuo: medio-alto.</t>
         </is>
@@ -1181,16 +1214,17 @@
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="6" t="n"/>
-      <c r="S9" s="4">
-        <f>IF(COUNT(K9:R9)=0,"",ROUND(SUMPRODUCT(K9:R9,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T9" s="6" t="inlineStr">
+      <c r="S9" s="6" t="n"/>
+      <c r="T9" s="4">
+        <f>IF(COUNT(K9:S9)=0,"",ROUND(SUMPRODUCT(K9:S9,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U9" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U9" s="6" t="inlineStr">
+      <c r="V9" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Applicabile dal 01/08/2025. Stato di armonizzazione degli standard discordante tra le fonti. Vantaggio tuo: alto (RF).</t>
         </is>
@@ -1244,16 +1278,17 @@
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="6" t="n"/>
-      <c r="S10" s="4">
-        <f>IF(COUNT(K10:R10)=0,"",ROUND(SUMPRODUCT(K10:R10,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
+      <c r="S10" s="6" t="n"/>
+      <c r="T10" s="4">
+        <f>IF(COUNT(K10:S10)=0,"",ROUND(SUMPRODUCT(K10:S10,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U10" s="6" t="inlineStr">
+      <c r="V10" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Applicazione dal 20/01/2027; UCIMU chiede una proroga condizionata. Dettagli sulla documentazione tecnica non verificati.</t>
         </is>
@@ -1299,16 +1334,17 @@
       <c r="P11" s="6" t="n"/>
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="6" t="n"/>
-      <c r="S11" s="4">
-        <f>IF(COUNT(K11:R11)=0,"",ROUND(SUMPRODUCT(K11:R11,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
+      <c r="S11" s="6" t="n"/>
+      <c r="T11" s="4">
+        <f>IF(COUNT(K11:S11)=0,"",ROUND(SUMPRODUCT(K11:S11,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U11" s="6" t="inlineStr">
+      <c r="V11" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Trasparenza dal 02/08/2026; alto rischio rinviato a dicembre 2027 / agosto 2028 (accordo provvisorio del 07/05/2026, da verificare in Gazzetta UE). Domanda specifica debole.</t>
         </is>
@@ -1354,16 +1390,17 @@
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="6" t="n"/>
-      <c r="S12" s="4">
-        <f>IF(COUNT(K12:R12)=0,"",ROUND(SUMPRODUCT(K12:R12,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T12" s="6" t="inlineStr">
+      <c r="S12" s="6" t="n"/>
+      <c r="T12" s="4">
+        <f>IF(COUNT(K12:S12)=0,"",ROUND(SUMPRODUCT(K12:S12,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U12" s="6" t="inlineStr">
+      <c r="V12" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Stato del decreto di recepimento discordante tra le fonti (D.Lgs. 96/2026?). Report annuale dal 07/06/2027 per 250+ dipendenti. Il target è piccolo: poche aziende con 100+ dipendenti.</t>
         </is>
@@ -1409,16 +1446,17 @@
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
       <c r="R13" s="6" t="n"/>
-      <c r="S13" s="4">
-        <f>IF(COUNT(K13:R13)=0,"",ROUND(SUMPRODUCT(K13:R13,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T13" s="6" t="inlineStr">
+      <c r="S13" s="6" t="n"/>
+      <c r="T13" s="4">
+        <f>IF(COUNT(K13:S13)=0,"",ROUND(SUMPRODUCT(K13:S13,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U13" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U13" s="6" t="inlineStr">
+      <c r="V13" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Applicabile dal 12/08/2026; date di etichettatura discordanti (2026, 2027, 2028). Assolombarda ha attivato un desk dedicato.</t>
         </is>
@@ -1464,16 +1502,17 @@
       <c r="P14" s="6" t="n"/>
       <c r="Q14" s="6" t="n"/>
       <c r="R14" s="6" t="n"/>
-      <c r="S14" s="4">
-        <f>IF(COUNT(K14:R14)=0,"",ROUND(SUMPRODUCT(K14:R14,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T14" s="6" t="inlineStr">
+      <c r="S14" s="6" t="n"/>
+      <c r="T14" s="4">
+        <f>IF(COUNT(K14:S14)=0,"",ROUND(SUMPRODUCT(K14:S14,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U14" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U14" s="6" t="inlineStr">
+      <c r="V14" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Batterie dal 18/02/2027; tessile non ancora definito. Dominato da grandi fornitori e dagli atti delegati.</t>
         </is>
@@ -1519,16 +1558,17 @@
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="6" t="n"/>
       <c r="R15" s="6" t="n"/>
-      <c r="S15" s="4">
-        <f>IF(COUNT(K15:R15)=0,"",ROUND(SUMPRODUCT(K15:R15,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T15" s="6" t="inlineStr">
+      <c r="S15" s="6" t="n"/>
+      <c r="T15" s="4">
+        <f>IF(COUNT(K15:S15)=0,"",ROUND(SUMPRODUCT(K15:S15,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U15" s="6" t="inlineStr">
+      <c r="V15" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Obbligo dal 28/06/2025; piattaforma di segnalazione AgID dal 11/03/2026; sanzioni da verificare (nessun procedimento pubblico trovato a giugno 2026). Molti fornitori.</t>
         </is>
@@ -1582,16 +1622,17 @@
       <c r="P16" s="6" t="n"/>
       <c r="Q16" s="6" t="n"/>
       <c r="R16" s="6" t="n"/>
-      <c r="S16" s="4">
-        <f>IF(COUNT(K16:R16)=0,"",ROUND(SUMPRODUCT(K16:R16,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T16" s="6" t="inlineStr">
+      <c r="S16" s="6" t="n"/>
+      <c r="T16" s="4">
+        <f>IF(COUNT(K16:S16)=0,"",ROUND(SUMPRODUCT(K16:S16,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U16" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U16" s="6" t="inlineStr">
+      <c r="V16" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Piattaforma GSE dal 12/06/2026; comunicazione di completamento entro 15/11/2028. La perizia è di un ingegnere iscritto all'albo: collegato agli studi che stai contattando. Regole (soglie, SaaS) discordanti tra le fonti.</t>
         </is>
@@ -1645,16 +1686,17 @@
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="6" t="n"/>
       <c r="R17" s="6" t="n"/>
-      <c r="S17" s="4">
-        <f>IF(COUNT(K17:R17)=0,"",ROUND(SUMPRODUCT(K17:R17,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T17" s="6" t="inlineStr">
+      <c r="S17" s="6" t="n"/>
+      <c r="T17" s="4">
+        <f>IF(COUNT(K17:S17)=0,"",ROUND(SUMPRODUCT(K17:S17,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U17" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U17" s="6" t="inlineStr">
+      <c r="V17" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Piano Italia 1 Giga in ritardo: 250–700 mila civici potrebbero uscire dal Piano. Committenti con portali propri; strumenti degli OTDR con report già inclusi.</t>
         </is>
@@ -1700,16 +1742,17 @@
       <c r="P18" s="6" t="n"/>
       <c r="Q18" s="6" t="n"/>
       <c r="R18" s="6" t="n"/>
-      <c r="S18" s="4">
-        <f>IF(COUNT(K18:R18)=0,"",ROUND(SUMPRODUCT(K18:R18,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T18" s="6" t="inlineStr">
+      <c r="S18" s="6" t="n"/>
+      <c r="T18" s="4">
+        <f>IF(COUNT(K18:S18)=0,"",ROUND(SUMPRODUCT(K18:S18,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U18" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U18" s="6" t="inlineStr">
+      <c r="V18" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Obiettivo di 15.000 CER a giugno 2026 probabilmente mancato; regole ancora instabili.</t>
         </is>
@@ -1755,16 +1798,17 @@
       <c r="P19" s="6" t="n"/>
       <c r="Q19" s="6" t="n"/>
       <c r="R19" s="6" t="n"/>
-      <c r="S19" s="4">
-        <f>IF(COUNT(K19:R19)=0,"",ROUND(SUMPRODUCT(K19:R19,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T19" s="6" t="inlineStr">
+      <c r="S19" s="6" t="n"/>
+      <c r="T19" s="4">
+        <f>IF(COUNT(K19:S19)=0,"",ROUND(SUMPRODUCT(K19:S19,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U19" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U19" s="6" t="inlineStr">
+      <c r="V19" s="6" t="inlineStr">
         <is>
           <t>Segnale da verificare: non cercato. Obbligo ricorrente (ogni 4 anni per le imprese soggette). Da verificare sulle norme e sul mercato.</t>
         </is>
@@ -1818,16 +1862,17 @@
       <c r="P20" s="6" t="n"/>
       <c r="Q20" s="6" t="n"/>
       <c r="R20" s="6" t="n"/>
-      <c r="S20" s="4">
-        <f>IF(COUNT(K20:R20)=0,"",ROUND(SUMPRODUCT(K20:R20,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T20" s="6" t="inlineStr">
+      <c r="S20" s="6" t="n"/>
+      <c r="T20" s="4">
+        <f>IF(COUNT(K20:S20)=0,"",ROUND(SUMPRODUCT(K20:S20,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U20" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U20" s="6" t="inlineStr">
+      <c r="V20" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Oltre 2,7 milioni di linee FWA, +13% in un anno; frequenze 26 GHz in assegnazione. Nessun dato recente sul numero di piccoli provider.</t>
         </is>
@@ -1873,16 +1918,17 @@
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="6" t="n"/>
       <c r="R21" s="6" t="n"/>
-      <c r="S21" s="4">
-        <f>IF(COUNT(K21:R21)=0,"",ROUND(SUMPRODUCT(K21:R21,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T21" s="6" t="inlineStr">
+      <c r="S21" s="6" t="n"/>
+      <c r="T21" s="4">
+        <f>IF(COUNT(K21:S21)=0,"",ROUND(SUMPRODUCT(K21:S21,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U21" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U21" s="6" t="inlineStr">
+      <c r="V21" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata. Vantaggio tuo alto; modello a risparmio condiviso. Da verificare quanto si risparmia davvero.</t>
         </is>
@@ -1912,9 +1958,17 @@
           <t>Aventis Advisors (Zucchetti)</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="10" t="n"/>
+      <c r="F22" s="10" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: magazzinaggio e supporto ai trasporti (52) con 10+ = 7.223; 52.10 e 52.29 con 10+ = 4.123 (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>3000</v>
+      </c>
       <c r="I22" s="11">
         <f>IF(H22&gt;0,ROUND(1000000/H22,0),"")</f>
         <v/>
@@ -1928,16 +1982,17 @@
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="6" t="n"/>
       <c r="R22" s="6" t="n"/>
-      <c r="S22" s="4">
-        <f>IF(COUNT(K22:R22)=0,"",ROUND(SUMPRODUCT(K22:R22,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T22" s="6" t="inlineStr">
+      <c r="S22" s="6" t="n"/>
+      <c r="T22" s="4">
+        <f>IF(COUNT(K22:S22)=0,"",ROUND(SUMPRODUCT(K22:S22,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U22" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U22" s="6" t="inlineStr">
+      <c r="V22" s="6" t="inlineStr">
         <is>
           <t>Zucchetti ha acquisito la maggioranza di AWMS (personale per fabbriche e logistica): segnale che il verticale vale. In zona: 6 imprese di conto terzi nell'elenco. Software di turni già presenti.</t>
         </is>
@@ -1967,9 +2022,17 @@
           <t>Aventis Advisors (TeamSystem)</t>
         </is>
       </c>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="10" t="n"/>
+      <c r="F23" s="10" t="n">
+        <v>16400</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 25 con 10+ = 16.356 (25.62 meccanica generale: 4.975); alto = + 28 con 10+ (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>2400</v>
+      </c>
       <c r="I23" s="11">
         <f>IF(H23&gt;0,ROUND(1000000/H23,0),"")</f>
         <v/>
@@ -1983,16 +2046,17 @@
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="6" t="n"/>
       <c r="R23" s="6" t="n"/>
-      <c r="S23" s="4">
-        <f>IF(COUNT(K23:R23)=0,"",ROUND(SUMPRODUCT(K23:R23,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T23" s="6" t="inlineStr">
+      <c r="S23" s="6" t="n"/>
+      <c r="T23" s="4">
+        <f>IF(COUNT(K23:S23)=0,"",ROUND(SUMPRODUCT(K23:S23,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U23" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U23" s="6" t="inlineStr">
+      <c r="V23" s="6" t="inlineStr">
         <is>
           <t>TeamSystem ha fatto 7 acquisizioni nel comparto industria/costruzioni/real estate: segnale di valore del verticale. Mercato presidiato da gruppi grandi.</t>
         </is>
@@ -2038,16 +2102,17 @@
       <c r="P24" s="6" t="n"/>
       <c r="Q24" s="6" t="n"/>
       <c r="R24" s="6" t="n"/>
-      <c r="S24" s="4">
-        <f>IF(COUNT(K24:R24)=0,"",ROUND(SUMPRODUCT(K24:R24,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T24" s="6" t="inlineStr">
+      <c r="S24" s="6" t="n"/>
+      <c r="T24" s="4">
+        <f>IF(COUNT(K24:S24)=0,"",ROUND(SUMPRODUCT(K24:S24,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U24" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U24" s="6" t="inlineStr">
+      <c r="V24" s="6" t="inlineStr">
         <is>
           <t>5 acquisizioni TeamSystem in legal/compliance/sicurezza. Prodotti già esistenti; da mappare i concorrenti.</t>
         </is>
@@ -2101,16 +2166,17 @@
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="6" t="n"/>
       <c r="R25" s="6" t="n"/>
-      <c r="S25" s="4">
-        <f>IF(COUNT(K25:R25)=0,"",ROUND(SUMPRODUCT(K25:R25,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T25" s="6" t="inlineStr">
+      <c r="S25" s="6" t="n"/>
+      <c r="T25" s="4">
+        <f>IF(COUNT(K25:S25)=0,"",ROUND(SUMPRODUCT(K25:S25,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U25" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U25" s="6" t="inlineStr">
+      <c r="V25" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata. Gli strumenti hanno già software di report. Vantaggio tuo: alto.</t>
         </is>
@@ -2156,16 +2222,17 @@
       <c r="P26" s="6" t="n"/>
       <c r="Q26" s="6" t="n"/>
       <c r="R26" s="6" t="n"/>
-      <c r="S26" s="4">
-        <f>IF(COUNT(K26:R26)=0,"",ROUND(SUMPRODUCT(K26:R26,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T26" s="6" t="inlineStr">
+      <c r="S26" s="6" t="n"/>
+      <c r="T26" s="4">
+        <f>IF(COUNT(K26:S26)=0,"",ROUND(SUMPRODUCT(K26:S26,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U26" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U26" s="6" t="inlineStr">
+      <c r="V26" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata.</t>
         </is>
@@ -2195,9 +2262,17 @@
           <t>idea precedente</t>
         </is>
       </c>
-      <c r="F27" s="10" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="10" t="n"/>
+      <c r="F27" s="10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: ingrosso di macchinari (466) e prodotti specializzati (467) con 10+ = 8.028; alto = + 25.62 (4.975) (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>1800</v>
+      </c>
       <c r="I27" s="11">
         <f>IF(H27&gt;0,ROUND(1000000/H27,0),"")</f>
         <v/>
@@ -2211,16 +2286,17 @@
       <c r="P27" s="6" t="n"/>
       <c r="Q27" s="6" t="n"/>
       <c r="R27" s="6" t="n"/>
-      <c r="S27" s="4">
-        <f>IF(COUNT(K27:R27)=0,"",ROUND(SUMPRODUCT(K27:R27,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T27" s="6" t="inlineStr">
+      <c r="S27" s="6" t="n"/>
+      <c r="T27" s="4">
+        <f>IF(COUNT(K27:S27)=0,"",ROUND(SUMPRODUCT(K27:S27,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U27" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U27" s="6" t="inlineStr">
+      <c r="V27" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata. Probabile presenza di gestionali; da verificare.</t>
         </is>
@@ -2250,9 +2326,17 @@
           <t>da cercare</t>
         </is>
       </c>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="10" t="n"/>
+      <c r="F28" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: come per gli incassi (ingrosso, metallo e macchinari con 10+) (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="n">
+        <v>1800</v>
+      </c>
       <c r="I28" s="11">
         <f>IF(H28&gt;0,ROUND(1000000/H28,0),"")</f>
         <v/>
@@ -2266,16 +2350,17 @@
       <c r="P28" s="6" t="n"/>
       <c r="Q28" s="6" t="n"/>
       <c r="R28" s="6" t="n"/>
-      <c r="S28" s="4">
-        <f>IF(COUNT(K28:R28)=0,"",ROUND(SUMPRODUCT(K28:R28,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T28" s="6" t="inlineStr">
+      <c r="S28" s="6" t="n"/>
+      <c r="T28" s="4">
+        <f>IF(COUNT(K28:S28)=0,"",ROUND(SUMPRODUCT(K28:S28,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U28" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U28" s="6" t="inlineStr">
+      <c r="V28" s="6" t="inlineStr">
         <is>
           <t>Segnale da verificare: non cercato. Da cercare tra gli annunci per ruoli ripetitivi (ufficio ordini, data entry).</t>
         </is>
@@ -2305,9 +2390,17 @@
           <t>idea Gemini</t>
         </is>
       </c>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="10" t="n"/>
+      <c r="F29" s="10" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 28: 9.059 con 10+, 2.179 con 50+, 22.720 totali (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="n">
+        <v>3000</v>
+      </c>
       <c r="I29" s="11">
         <f>IF(H29&gt;0,ROUND(1000000/H29,0),"")</f>
         <v/>
@@ -2321,16 +2414,17 @@
       <c r="P29" s="6" t="n"/>
       <c r="Q29" s="6" t="n"/>
       <c r="R29" s="6" t="n"/>
-      <c r="S29" s="4">
-        <f>IF(COUNT(K29:R29)=0,"",ROUND(SUMPRODUCT(K29:R29,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T29" s="6" t="inlineStr">
+      <c r="S29" s="6" t="n"/>
+      <c r="T29" s="4">
+        <f>IF(COUNT(K29:S29)=0,"",ROUND(SUMPRODUCT(K29:S29,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U29" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U29" s="6" t="inlineStr">
+      <c r="V29" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata.</t>
         </is>
@@ -2376,16 +2470,17 @@
       <c r="P30" s="6" t="n"/>
       <c r="Q30" s="6" t="n"/>
       <c r="R30" s="6" t="n"/>
-      <c r="S30" s="4">
-        <f>IF(COUNT(K30:R30)=0,"",ROUND(SUMPRODUCT(K30:R30,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T30" s="6" t="inlineStr">
+      <c r="S30" s="6" t="n"/>
+      <c r="T30" s="4">
+        <f>IF(COUNT(K30:S30)=0,"",ROUND(SUMPRODUCT(K30:S30,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U30" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U30" s="6" t="inlineStr">
+      <c r="V30" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata. Gli studi (DEAL, Parodi, Lommano) fanno pratiche antincendio, certificazioni energetiche, perizie.</t>
         </is>
@@ -2431,16 +2526,17 @@
       <c r="P31" s="6" t="n"/>
       <c r="Q31" s="6" t="n"/>
       <c r="R31" s="6" t="n"/>
-      <c r="S31" s="4">
-        <f>IF(COUNT(K31:R31)=0,"",ROUND(SUMPRODUCT(K31:R31,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T31" s="6" t="inlineStr">
+      <c r="S31" s="6" t="n"/>
+      <c r="T31" s="4">
+        <f>IF(COUNT(K31:S31)=0,"",ROUND(SUMPRODUCT(K31:S31,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U31" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U31" s="6" t="inlineStr">
+      <c r="V31" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata. Vantaggio tuo: alto.</t>
         </is>
@@ -2486,16 +2582,17 @@
       <c r="P32" s="6" t="n"/>
       <c r="Q32" s="6" t="n"/>
       <c r="R32" s="6" t="n"/>
-      <c r="S32" s="4">
-        <f>IF(COUNT(K32:R32)=0,"",ROUND(SUMPRODUCT(K32:R32,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T32" s="6" t="inlineStr">
+      <c r="S32" s="6" t="n"/>
+      <c r="T32" s="4">
+        <f>IF(COUNT(K32:S32)=0,"",ROUND(SUMPRODUCT(K32:S32,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U32" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U32" s="6" t="inlineStr">
+      <c r="V32" s="6" t="inlineStr">
         <is>
           <t>Segnale da verificare: non cercato.</t>
         </is>
@@ -2541,16 +2638,17 @@
       <c r="P33" s="6" t="n"/>
       <c r="Q33" s="6" t="n"/>
       <c r="R33" s="6" t="n"/>
-      <c r="S33" s="4">
-        <f>IF(COUNT(K33:R33)=0,"",ROUND(SUMPRODUCT(K33:R33,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T33" s="6" t="inlineStr">
+      <c r="S33" s="6" t="n"/>
+      <c r="T33" s="4">
+        <f>IF(COUNT(K33:S33)=0,"",ROUND(SUMPRODUCT(K33:S33,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U33" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U33" s="6" t="inlineStr">
+      <c r="V33" s="6" t="inlineStr">
         <is>
           <t>Segnale da verificare: non cercato. Barriera regolatoria alta (GMP).</t>
         </is>
@@ -2596,16 +2694,17 @@
       <c r="P34" s="6" t="n"/>
       <c r="Q34" s="6" t="n"/>
       <c r="R34" s="6" t="n"/>
-      <c r="S34" s="4">
-        <f>IF(COUNT(K34:R34)=0,"",ROUND(SUMPRODUCT(K34:R34,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T34" s="6" t="inlineStr">
+      <c r="S34" s="6" t="n"/>
+      <c r="T34" s="4">
+        <f>IF(COUNT(K34:S34)=0,"",ROUND(SUMPRODUCT(K34:S34,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U34" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U34" s="6" t="inlineStr">
+      <c r="V34" s="6" t="inlineStr">
         <is>
           <t>Segnale verificato in ricerca (stampa di settore). Mercato affollato e a basso prezzo.</t>
         </is>
@@ -2651,16 +2750,17 @@
       <c r="P35" s="6" t="n"/>
       <c r="Q35" s="6" t="n"/>
       <c r="R35" s="6" t="n"/>
-      <c r="S35" s="4">
-        <f>IF(COUNT(K35:R35)=0,"",ROUND(SUMPRODUCT(K35:R35,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T35" s="6" t="inlineStr">
+      <c r="S35" s="6" t="n"/>
+      <c r="T35" s="4">
+        <f>IF(COUNT(K35:S35)=0,"",ROUND(SUMPRODUCT(K35:S35,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U35" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U35" s="6" t="inlineStr">
+      <c r="V35" s="6" t="inlineStr">
         <is>
           <t>Solo ipotesi nostra: domanda non verificata. Concorrenza forte (grandi fornitori).</t>
         </is>
@@ -2672,27 +2772,35 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Gestione documentale per sicurezza prodotti (GPSR) di importatori e venditori online</t>
+          <t>Incassi e solleciti: gestione automatica del credito e previsione di cassa per PMI B2B</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Importatori e e-commerce di prodotti per consumatori</t>
+          <t>PMI B2B (ingrosso, manifattura) con molte fatture</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Obbligo di legge</t>
+          <t>Ritardi di pagamento</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>da cercare</t>
-        </is>
-      </c>
-      <c r="F36" s="10" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="10" t="n"/>
+          <t>Cribis; Cerved; Intrum</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: unità locali con 10+ addetti in ingrosso (46: 20.256), metallo (25: 16.356), macchinari (28: 9.059); basso = 50+ (5.804). Cribis 2026: solo 42% paga puntuale (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H36" s="10" t="n">
+        <v>1200</v>
+      </c>
       <c r="I36" s="11">
         <f>IF(H36&gt;0,ROUND(1000000/H36,0),"")</f>
         <v/>
@@ -2706,32 +2814,57 @@
       <c r="P36" s="6" t="n"/>
       <c r="Q36" s="6" t="n"/>
       <c r="R36" s="6" t="n"/>
-      <c r="S36" s="4">
-        <f>IF(COUNT(K36:R36)=0,"",ROUND(SUMPRODUCT(K36:R36,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T36" s="6" t="inlineStr">
+      <c r="S36" s="6" t="n"/>
+      <c r="T36" s="4">
+        <f>IF(COUNT(K36:S36)=0,"",ROUND(SUMPRODUCT(K36:S36,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U36" s="6" t="inlineStr">
         <is>
           <t>Da studiare</t>
         </is>
       </c>
-      <c r="U36" s="6" t="inlineStr">
-        <is>
-          <t>Segnale da verificare: non cercato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
+      <c r="V36" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). Cribis giugno 2026: solo il 42% delle imprese paga puntuale (piccole 41,8%, medie 35,7%, grandi 21,1%). Intrum 2024: ~81 giorni di incasso medi in Italia contro ~50 in Europa. Bisogno di cassa permanente. Concorrenza alta (gestionali, fintech).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="92" customHeight="1">
       <c r="A37" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="10" t="n"/>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="10" t="n"/>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>TMS leggero per piccole imprese di autotrasporto (DDT/CMR, scadenze, pianificazione)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Autotrasportatori conto terzi</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Dolore operativo permanente</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Uomini e Trasporti; Istat</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 49.41 = 63.633 unità locali, 9.037 con 10+, 915 con 50+; alto = 10+ più 25% delle micro (mia ipotesi). Imprese attive in calo del 22% dal 2015 (affidabilità: Media-bassa)</t>
+        </is>
+      </c>
+      <c r="H37" s="10" t="n">
+        <v>1200</v>
+      </c>
       <c r="I37" s="11">
         <f>IF(H37&gt;0,ROUND(1000000/H37,0),"")</f>
         <v/>
@@ -2745,24 +2878,57 @@
       <c r="P37" s="6" t="n"/>
       <c r="Q37" s="6" t="n"/>
       <c r="R37" s="6" t="n"/>
-      <c r="S37" s="4">
-        <f>IF(COUNT(K37:R37)=0,"",ROUND(SUMPRODUCT(K37:R37,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T37" s="6" t="n"/>
-      <c r="U37" s="6" t="n"/>
-    </row>
-    <row r="38">
+      <c r="S37" s="6" t="n"/>
+      <c r="T37" s="4">
+        <f>IF(COUNT(K37:S37)=0,"",ROUND(SUMPRODUCT(K37:S37,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U37" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="V37" s="6" t="inlineStr">
+        <is>
+          <t>Segnale verificato in ricerca (stampa di settore). 67.349 imprese attive nel 2025 (-22% dal 2015), le ditte individuali -41%: il settore si concentra, i clienti diminuiscono. Il cugino della tua ragazza ha una ditta di trasporti: possibile primo contatto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="92" customHeight="1">
       <c r="A38" s="9" t="n">
         <v>33</v>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="10" t="n"/>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Spedizionieri e magazzini: documenti, tracciamento e dogane</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Spedizionieri, operatori logistici</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Dolore operativo permanente</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Istat</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 52.29 e 52.10 con 10+ = 4.123; 50+ = 849; alto = 52.2 con 10+ (6.583) (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H38" s="10" t="n">
+        <v>2400</v>
+      </c>
       <c r="I38" s="11">
         <f>IF(H38&gt;0,ROUND(1000000/H38,0),"")</f>
         <v/>
@@ -2776,24 +2942,57 @@
       <c r="P38" s="6" t="n"/>
       <c r="Q38" s="6" t="n"/>
       <c r="R38" s="6" t="n"/>
-      <c r="S38" s="4">
-        <f>IF(COUNT(K38:R38)=0,"",ROUND(SUMPRODUCT(K38:R38,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T38" s="6" t="n"/>
-      <c r="U38" s="6" t="n"/>
-    </row>
-    <row r="39">
+      <c r="S38" s="6" t="n"/>
+      <c r="T38" s="4">
+        <f>IF(COUNT(K38:S38)=0,"",ROUND(SUMPRODUCT(K38:S38,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U38" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="V38" s="6" t="inlineStr">
+        <is>
+          <t>Mercato medio (ATECO 52.29 e 52.10). Segnale da verificare: non cercato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="92" customHeight="1">
       <c r="A39" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="10" t="n"/>
-      <c r="G39" s="6" t="n"/>
-      <c r="H39" s="10" t="n"/>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Gestione commesse e tracciabilità per officine e subfornitura meccanica</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Officine meccaniche e carpenterie con 10+ addetti</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Dolore operativo permanente</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Istat</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>16400</v>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 25 con 10+ = 16.356 (25.62 meccanica generale: 4.975); alto = + 28 con 10+ (affidabilità: Media)</t>
+        </is>
+      </c>
+      <c r="H39" s="10" t="n">
+        <v>2400</v>
+      </c>
       <c r="I39" s="11">
         <f>IF(H39&gt;0,ROUND(1000000/H39,0),"")</f>
         <v/>
@@ -2807,21 +3006,46 @@
       <c r="P39" s="6" t="n"/>
       <c r="Q39" s="6" t="n"/>
       <c r="R39" s="6" t="n"/>
-      <c r="S39" s="4">
-        <f>IF(COUNT(K39:R39)=0,"",ROUND(SUMPRODUCT(K39:R39,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T39" s="6" t="n"/>
-      <c r="U39" s="6" t="n"/>
-    </row>
-    <row r="40">
+      <c r="S39" s="6" t="n"/>
+      <c r="T39" s="4">
+        <f>IF(COUNT(K39:S39)=0,"",ROUND(SUMPRODUCT(K39:S39,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U39" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="V39" s="6" t="inlineStr">
+        <is>
+          <t>Solo ipotesi nostra: domanda non verificata. Richiede conoscenza del mestiere; presenti ERP e MES.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="92" customHeight="1">
       <c r="A40" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Export: documentazione per PMI esportatrici (origine, dogana)</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>PMI esportatrici</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Dolore operativo permanente</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Istat-ICE 2025</t>
+        </is>
+      </c>
       <c r="F40" s="10" t="n"/>
       <c r="G40" s="6" t="n"/>
       <c r="H40" s="10" t="n"/>
@@ -2838,21 +3062,46 @@
       <c r="P40" s="6" t="n"/>
       <c r="Q40" s="6" t="n"/>
       <c r="R40" s="6" t="n"/>
-      <c r="S40" s="4">
-        <f>IF(COUNT(K40:R40)=0,"",ROUND(SUMPRODUCT(K40:R40,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T40" s="6" t="n"/>
-      <c r="U40" s="6" t="n"/>
-    </row>
-    <row r="41">
+      <c r="S40" s="6" t="n"/>
+      <c r="T40" s="4">
+        <f>IF(COUNT(K40:S40)=0,"",ROUND(SUMPRODUCT(K40:S40,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U40" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="V40" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato. 120.170 imprese esportatrici attive nel 2023; nessun dato su costo della documentazione.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="92" customHeight="1">
       <c r="A41" s="9" t="n">
         <v>36</v>
       </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Gestione documentale per sicurezza prodotti (GPSR) di importatori e venditori online</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Importatori e e-commerce di prodotti per consumatori</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di legge</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>da cercare</t>
+        </is>
+      </c>
       <c r="F41" s="10" t="n"/>
       <c r="G41" s="6" t="n"/>
       <c r="H41" s="10" t="n"/>
@@ -2869,12 +3118,21 @@
       <c r="P41" s="6" t="n"/>
       <c r="Q41" s="6" t="n"/>
       <c r="R41" s="6" t="n"/>
-      <c r="S41" s="4">
-        <f>IF(COUNT(K41:R41)=0,"",ROUND(SUMPRODUCT(K41:R41,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T41" s="6" t="n"/>
-      <c r="U41" s="6" t="n"/>
+      <c r="S41" s="6" t="n"/>
+      <c r="T41" s="4">
+        <f>IF(COUNT(K41:S41)=0,"",ROUND(SUMPRODUCT(K41:S41,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
+      <c r="U41" s="6" t="inlineStr">
+        <is>
+          <t>Da studiare</t>
+        </is>
+      </c>
+      <c r="V41" s="6" t="inlineStr">
+        <is>
+          <t>Segnale da verificare: non cercato.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n">
@@ -2900,12 +3158,13 @@
       <c r="P42" s="6" t="n"/>
       <c r="Q42" s="6" t="n"/>
       <c r="R42" s="6" t="n"/>
-      <c r="S42" s="4">
-        <f>IF(COUNT(K42:R42)=0,"",ROUND(SUMPRODUCT(K42:R42,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T42" s="6" t="n"/>
+      <c r="S42" s="6" t="n"/>
+      <c r="T42" s="4">
+        <f>IF(COUNT(K42:S42)=0,"",ROUND(SUMPRODUCT(K42:S42,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U42" s="6" t="n"/>
+      <c r="V42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
@@ -2931,12 +3190,13 @@
       <c r="P43" s="6" t="n"/>
       <c r="Q43" s="6" t="n"/>
       <c r="R43" s="6" t="n"/>
-      <c r="S43" s="4">
-        <f>IF(COUNT(K43:R43)=0,"",ROUND(SUMPRODUCT(K43:R43,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T43" s="6" t="n"/>
+      <c r="S43" s="6" t="n"/>
+      <c r="T43" s="4">
+        <f>IF(COUNT(K43:S43)=0,"",ROUND(SUMPRODUCT(K43:S43,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U43" s="6" t="n"/>
+      <c r="V43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n">
@@ -2962,12 +3222,13 @@
       <c r="P44" s="6" t="n"/>
       <c r="Q44" s="6" t="n"/>
       <c r="R44" s="6" t="n"/>
-      <c r="S44" s="4">
-        <f>IF(COUNT(K44:R44)=0,"",ROUND(SUMPRODUCT(K44:R44,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T44" s="6" t="n"/>
+      <c r="S44" s="6" t="n"/>
+      <c r="T44" s="4">
+        <f>IF(COUNT(K44:S44)=0,"",ROUND(SUMPRODUCT(K44:S44,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U44" s="6" t="n"/>
+      <c r="V44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n">
@@ -2993,12 +3254,13 @@
       <c r="P45" s="6" t="n"/>
       <c r="Q45" s="6" t="n"/>
       <c r="R45" s="6" t="n"/>
-      <c r="S45" s="4">
-        <f>IF(COUNT(K45:R45)=0,"",ROUND(SUMPRODUCT(K45:R45,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T45" s="6" t="n"/>
+      <c r="S45" s="6" t="n"/>
+      <c r="T45" s="4">
+        <f>IF(COUNT(K45:S45)=0,"",ROUND(SUMPRODUCT(K45:S45,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U45" s="6" t="n"/>
+      <c r="V45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n">
@@ -3024,12 +3286,13 @@
       <c r="P46" s="6" t="n"/>
       <c r="Q46" s="6" t="n"/>
       <c r="R46" s="6" t="n"/>
-      <c r="S46" s="4">
-        <f>IF(COUNT(K46:R46)=0,"",ROUND(SUMPRODUCT(K46:R46,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T46" s="6" t="n"/>
+      <c r="S46" s="6" t="n"/>
+      <c r="T46" s="4">
+        <f>IF(COUNT(K46:S46)=0,"",ROUND(SUMPRODUCT(K46:S46,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U46" s="6" t="n"/>
+      <c r="V46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
@@ -3055,12 +3318,13 @@
       <c r="P47" s="6" t="n"/>
       <c r="Q47" s="6" t="n"/>
       <c r="R47" s="6" t="n"/>
-      <c r="S47" s="4">
-        <f>IF(COUNT(K47:R47)=0,"",ROUND(SUMPRODUCT(K47:R47,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T47" s="6" t="n"/>
+      <c r="S47" s="6" t="n"/>
+      <c r="T47" s="4">
+        <f>IF(COUNT(K47:S47)=0,"",ROUND(SUMPRODUCT(K47:S47,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U47" s="6" t="n"/>
+      <c r="V47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
@@ -3086,12 +3350,13 @@
       <c r="P48" s="6" t="n"/>
       <c r="Q48" s="6" t="n"/>
       <c r="R48" s="6" t="n"/>
-      <c r="S48" s="4">
-        <f>IF(COUNT(K48:R48)=0,"",ROUND(SUMPRODUCT(K48:R48,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T48" s="6" t="n"/>
+      <c r="S48" s="6" t="n"/>
+      <c r="T48" s="4">
+        <f>IF(COUNT(K48:S48)=0,"",ROUND(SUMPRODUCT(K48:S48,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U48" s="6" t="n"/>
+      <c r="V48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
@@ -3117,12 +3382,13 @@
       <c r="P49" s="6" t="n"/>
       <c r="Q49" s="6" t="n"/>
       <c r="R49" s="6" t="n"/>
-      <c r="S49" s="4">
-        <f>IF(COUNT(K49:R49)=0,"",ROUND(SUMPRODUCT(K49:R49,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T49" s="6" t="n"/>
+      <c r="S49" s="6" t="n"/>
+      <c r="T49" s="4">
+        <f>IF(COUNT(K49:S49)=0,"",ROUND(SUMPRODUCT(K49:S49,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U49" s="6" t="n"/>
+      <c r="V49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
@@ -3148,12 +3414,13 @@
       <c r="P50" s="6" t="n"/>
       <c r="Q50" s="6" t="n"/>
       <c r="R50" s="6" t="n"/>
-      <c r="S50" s="4">
-        <f>IF(COUNT(K50:R50)=0,"",ROUND(SUMPRODUCT(K50:R50,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T50" s="6" t="n"/>
+      <c r="S50" s="6" t="n"/>
+      <c r="T50" s="4">
+        <f>IF(COUNT(K50:S50)=0,"",ROUND(SUMPRODUCT(K50:S50,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U50" s="6" t="n"/>
+      <c r="V50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
@@ -3179,12 +3446,13 @@
       <c r="P51" s="6" t="n"/>
       <c r="Q51" s="6" t="n"/>
       <c r="R51" s="6" t="n"/>
-      <c r="S51" s="4">
-        <f>IF(COUNT(K51:R51)=0,"",ROUND(SUMPRODUCT(K51:R51,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T51" s="6" t="n"/>
+      <c r="S51" s="6" t="n"/>
+      <c r="T51" s="4">
+        <f>IF(COUNT(K51:S51)=0,"",ROUND(SUMPRODUCT(K51:S51,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U51" s="6" t="n"/>
+      <c r="V51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="9" t="n">
@@ -3210,12 +3478,13 @@
       <c r="P52" s="6" t="n"/>
       <c r="Q52" s="6" t="n"/>
       <c r="R52" s="6" t="n"/>
-      <c r="S52" s="4">
-        <f>IF(COUNT(K52:R52)=0,"",ROUND(SUMPRODUCT(K52:R52,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T52" s="6" t="n"/>
+      <c r="S52" s="6" t="n"/>
+      <c r="T52" s="4">
+        <f>IF(COUNT(K52:S52)=0,"",ROUND(SUMPRODUCT(K52:S52,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U52" s="6" t="n"/>
+      <c r="V52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
@@ -3241,12 +3510,13 @@
       <c r="P53" s="6" t="n"/>
       <c r="Q53" s="6" t="n"/>
       <c r="R53" s="6" t="n"/>
-      <c r="S53" s="4">
-        <f>IF(COUNT(K53:R53)=0,"",ROUND(SUMPRODUCT(K53:R53,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T53" s="6" t="n"/>
+      <c r="S53" s="6" t="n"/>
+      <c r="T53" s="4">
+        <f>IF(COUNT(K53:S53)=0,"",ROUND(SUMPRODUCT(K53:S53,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U53" s="6" t="n"/>
+      <c r="V53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n">
@@ -3272,12 +3542,13 @@
       <c r="P54" s="6" t="n"/>
       <c r="Q54" s="6" t="n"/>
       <c r="R54" s="6" t="n"/>
-      <c r="S54" s="4">
-        <f>IF(COUNT(K54:R54)=0,"",ROUND(SUMPRODUCT(K54:R54,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T54" s="6" t="n"/>
+      <c r="S54" s="6" t="n"/>
+      <c r="T54" s="4">
+        <f>IF(COUNT(K54:S54)=0,"",ROUND(SUMPRODUCT(K54:S54,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U54" s="6" t="n"/>
+      <c r="V54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
@@ -3303,12 +3574,13 @@
       <c r="P55" s="6" t="n"/>
       <c r="Q55" s="6" t="n"/>
       <c r="R55" s="6" t="n"/>
-      <c r="S55" s="4">
-        <f>IF(COUNT(K55:R55)=0,"",ROUND(SUMPRODUCT(K55:R55,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T55" s="6" t="n"/>
+      <c r="S55" s="6" t="n"/>
+      <c r="T55" s="4">
+        <f>IF(COUNT(K55:S55)=0,"",ROUND(SUMPRODUCT(K55:S55,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U55" s="6" t="n"/>
+      <c r="V55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
@@ -3334,12 +3606,13 @@
       <c r="P56" s="6" t="n"/>
       <c r="Q56" s="6" t="n"/>
       <c r="R56" s="6" t="n"/>
-      <c r="S56" s="4">
-        <f>IF(COUNT(K56:R56)=0,"",ROUND(SUMPRODUCT(K56:R56,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T56" s="6" t="n"/>
+      <c r="S56" s="6" t="n"/>
+      <c r="T56" s="4">
+        <f>IF(COUNT(K56:S56)=0,"",ROUND(SUMPRODUCT(K56:S56,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U56" s="6" t="n"/>
+      <c r="V56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
@@ -3365,12 +3638,13 @@
       <c r="P57" s="6" t="n"/>
       <c r="Q57" s="6" t="n"/>
       <c r="R57" s="6" t="n"/>
-      <c r="S57" s="4">
-        <f>IF(COUNT(K57:R57)=0,"",ROUND(SUMPRODUCT(K57:R57,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T57" s="6" t="n"/>
+      <c r="S57" s="6" t="n"/>
+      <c r="T57" s="4">
+        <f>IF(COUNT(K57:S57)=0,"",ROUND(SUMPRODUCT(K57:S57,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U57" s="6" t="n"/>
+      <c r="V57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
@@ -3396,12 +3670,13 @@
       <c r="P58" s="6" t="n"/>
       <c r="Q58" s="6" t="n"/>
       <c r="R58" s="6" t="n"/>
-      <c r="S58" s="4">
-        <f>IF(COUNT(K58:R58)=0,"",ROUND(SUMPRODUCT(K58:R58,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T58" s="6" t="n"/>
+      <c r="S58" s="6" t="n"/>
+      <c r="T58" s="4">
+        <f>IF(COUNT(K58:S58)=0,"",ROUND(SUMPRODUCT(K58:S58,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U58" s="6" t="n"/>
+      <c r="V58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n">
@@ -3427,12 +3702,13 @@
       <c r="P59" s="6" t="n"/>
       <c r="Q59" s="6" t="n"/>
       <c r="R59" s="6" t="n"/>
-      <c r="S59" s="4">
-        <f>IF(COUNT(K59:R59)=0,"",ROUND(SUMPRODUCT(K59:R59,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T59" s="6" t="n"/>
+      <c r="S59" s="6" t="n"/>
+      <c r="T59" s="4">
+        <f>IF(COUNT(K59:S59)=0,"",ROUND(SUMPRODUCT(K59:S59,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U59" s="6" t="n"/>
+      <c r="V59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n">
@@ -3458,12 +3734,13 @@
       <c r="P60" s="6" t="n"/>
       <c r="Q60" s="6" t="n"/>
       <c r="R60" s="6" t="n"/>
-      <c r="S60" s="4">
-        <f>IF(COUNT(K60:R60)=0,"",ROUND(SUMPRODUCT(K60:R60,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T60" s="6" t="n"/>
+      <c r="S60" s="6" t="n"/>
+      <c r="T60" s="4">
+        <f>IF(COUNT(K60:S60)=0,"",ROUND(SUMPRODUCT(K60:S60,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U60" s="6" t="n"/>
+      <c r="V60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
@@ -3489,12 +3766,13 @@
       <c r="P61" s="6" t="n"/>
       <c r="Q61" s="6" t="n"/>
       <c r="R61" s="6" t="n"/>
-      <c r="S61" s="4">
-        <f>IF(COUNT(K61:R61)=0,"",ROUND(SUMPRODUCT(K61:R61,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T61" s="6" t="n"/>
+      <c r="S61" s="6" t="n"/>
+      <c r="T61" s="4">
+        <f>IF(COUNT(K61:S61)=0,"",ROUND(SUMPRODUCT(K61:S61,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U61" s="6" t="n"/>
+      <c r="V61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
@@ -3520,12 +3798,13 @@
       <c r="P62" s="6" t="n"/>
       <c r="Q62" s="6" t="n"/>
       <c r="R62" s="6" t="n"/>
-      <c r="S62" s="4">
-        <f>IF(COUNT(K62:R62)=0,"",ROUND(SUMPRODUCT(K62:R62,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T62" s="6" t="n"/>
+      <c r="S62" s="6" t="n"/>
+      <c r="T62" s="4">
+        <f>IF(COUNT(K62:S62)=0,"",ROUND(SUMPRODUCT(K62:S62,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U62" s="6" t="n"/>
+      <c r="V62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
@@ -3551,12 +3830,13 @@
       <c r="P63" s="6" t="n"/>
       <c r="Q63" s="6" t="n"/>
       <c r="R63" s="6" t="n"/>
-      <c r="S63" s="4">
-        <f>IF(COUNT(K63:R63)=0,"",ROUND(SUMPRODUCT(K63:R63,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T63" s="6" t="n"/>
+      <c r="S63" s="6" t="n"/>
+      <c r="T63" s="4">
+        <f>IF(COUNT(K63:S63)=0,"",ROUND(SUMPRODUCT(K63:S63,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U63" s="6" t="n"/>
+      <c r="V63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
@@ -3582,12 +3862,13 @@
       <c r="P64" s="6" t="n"/>
       <c r="Q64" s="6" t="n"/>
       <c r="R64" s="6" t="n"/>
-      <c r="S64" s="4">
-        <f>IF(COUNT(K64:R64)=0,"",ROUND(SUMPRODUCT(K64:R64,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T64" s="6" t="n"/>
+      <c r="S64" s="6" t="n"/>
+      <c r="T64" s="4">
+        <f>IF(COUNT(K64:S64)=0,"",ROUND(SUMPRODUCT(K64:S64,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U64" s="6" t="n"/>
+      <c r="V64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
@@ -3613,12 +3894,13 @@
       <c r="P65" s="6" t="n"/>
       <c r="Q65" s="6" t="n"/>
       <c r="R65" s="6" t="n"/>
-      <c r="S65" s="4">
-        <f>IF(COUNT(K65:R65)=0,"",ROUND(SUMPRODUCT(K65:R65,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T65" s="6" t="n"/>
+      <c r="S65" s="6" t="n"/>
+      <c r="T65" s="4">
+        <f>IF(COUNT(K65:S65)=0,"",ROUND(SUMPRODUCT(K65:S65,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U65" s="6" t="n"/>
+      <c r="V65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
@@ -3644,12 +3926,13 @@
       <c r="P66" s="6" t="n"/>
       <c r="Q66" s="6" t="n"/>
       <c r="R66" s="6" t="n"/>
-      <c r="S66" s="4">
-        <f>IF(COUNT(K66:R66)=0,"",ROUND(SUMPRODUCT(K66:R66,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T66" s="6" t="n"/>
+      <c r="S66" s="6" t="n"/>
+      <c r="T66" s="4">
+        <f>IF(COUNT(K66:S66)=0,"",ROUND(SUMPRODUCT(K66:S66,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U66" s="6" t="n"/>
+      <c r="V66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
@@ -3675,12 +3958,13 @@
       <c r="P67" s="6" t="n"/>
       <c r="Q67" s="6" t="n"/>
       <c r="R67" s="6" t="n"/>
-      <c r="S67" s="4">
-        <f>IF(COUNT(K67:R67)=0,"",ROUND(SUMPRODUCT(K67:R67,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T67" s="6" t="n"/>
+      <c r="S67" s="6" t="n"/>
+      <c r="T67" s="4">
+        <f>IF(COUNT(K67:S67)=0,"",ROUND(SUMPRODUCT(K67:S67,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U67" s="6" t="n"/>
+      <c r="V67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
@@ -3706,12 +3990,13 @@
       <c r="P68" s="6" t="n"/>
       <c r="Q68" s="6" t="n"/>
       <c r="R68" s="6" t="n"/>
-      <c r="S68" s="4">
-        <f>IF(COUNT(K68:R68)=0,"",ROUND(SUMPRODUCT(K68:R68,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T68" s="6" t="n"/>
+      <c r="S68" s="6" t="n"/>
+      <c r="T68" s="4">
+        <f>IF(COUNT(K68:S68)=0,"",ROUND(SUMPRODUCT(K68:S68,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U68" s="6" t="n"/>
+      <c r="V68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
@@ -3737,12 +4022,13 @@
       <c r="P69" s="6" t="n"/>
       <c r="Q69" s="6" t="n"/>
       <c r="R69" s="6" t="n"/>
-      <c r="S69" s="4">
-        <f>IF(COUNT(K69:R69)=0,"",ROUND(SUMPRODUCT(K69:R69,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T69" s="6" t="n"/>
+      <c r="S69" s="6" t="n"/>
+      <c r="T69" s="4">
+        <f>IF(COUNT(K69:S69)=0,"",ROUND(SUMPRODUCT(K69:S69,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U69" s="6" t="n"/>
+      <c r="V69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
@@ -3768,12 +4054,13 @@
       <c r="P70" s="6" t="n"/>
       <c r="Q70" s="6" t="n"/>
       <c r="R70" s="6" t="n"/>
-      <c r="S70" s="4">
-        <f>IF(COUNT(K70:R70)=0,"",ROUND(SUMPRODUCT(K70:R70,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T70" s="6" t="n"/>
+      <c r="S70" s="6" t="n"/>
+      <c r="T70" s="4">
+        <f>IF(COUNT(K70:S70)=0,"",ROUND(SUMPRODUCT(K70:S70,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U70" s="6" t="n"/>
+      <c r="V70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
@@ -3799,12 +4086,13 @@
       <c r="P71" s="6" t="n"/>
       <c r="Q71" s="6" t="n"/>
       <c r="R71" s="6" t="n"/>
-      <c r="S71" s="4">
-        <f>IF(COUNT(K71:R71)=0,"",ROUND(SUMPRODUCT(K71:R71,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T71" s="6" t="n"/>
+      <c r="S71" s="6" t="n"/>
+      <c r="T71" s="4">
+        <f>IF(COUNT(K71:S71)=0,"",ROUND(SUMPRODUCT(K71:S71,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U71" s="6" t="n"/>
+      <c r="V71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="9" t="n">
@@ -3830,12 +4118,13 @@
       <c r="P72" s="6" t="n"/>
       <c r="Q72" s="6" t="n"/>
       <c r="R72" s="6" t="n"/>
-      <c r="S72" s="4">
-        <f>IF(COUNT(K72:R72)=0,"",ROUND(SUMPRODUCT(K72:R72,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T72" s="6" t="n"/>
+      <c r="S72" s="6" t="n"/>
+      <c r="T72" s="4">
+        <f>IF(COUNT(K72:S72)=0,"",ROUND(SUMPRODUCT(K72:S72,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U72" s="6" t="n"/>
+      <c r="V72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n">
@@ -3861,12 +4150,13 @@
       <c r="P73" s="6" t="n"/>
       <c r="Q73" s="6" t="n"/>
       <c r="R73" s="6" t="n"/>
-      <c r="S73" s="4">
-        <f>IF(COUNT(K73:R73)=0,"",ROUND(SUMPRODUCT(K73:R73,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T73" s="6" t="n"/>
+      <c r="S73" s="6" t="n"/>
+      <c r="T73" s="4">
+        <f>IF(COUNT(K73:S73)=0,"",ROUND(SUMPRODUCT(K73:S73,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U73" s="6" t="n"/>
+      <c r="V73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
@@ -3892,12 +4182,13 @@
       <c r="P74" s="6" t="n"/>
       <c r="Q74" s="6" t="n"/>
       <c r="R74" s="6" t="n"/>
-      <c r="S74" s="4">
-        <f>IF(COUNT(K74:R74)=0,"",ROUND(SUMPRODUCT(K74:R74,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T74" s="6" t="n"/>
+      <c r="S74" s="6" t="n"/>
+      <c r="T74" s="4">
+        <f>IF(COUNT(K74:S74)=0,"",ROUND(SUMPRODUCT(K74:S74,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U74" s="6" t="n"/>
+      <c r="V74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
@@ -3923,26 +4214,27 @@
       <c r="P75" s="6" t="n"/>
       <c r="Q75" s="6" t="n"/>
       <c r="R75" s="6" t="n"/>
-      <c r="S75" s="4">
-        <f>IF(COUNT(K75:R75)=0,"",ROUND(SUMPRODUCT(K75:R75,K$4:R$4)/SUM(K$4:R$4),2))</f>
-        <v/>
-      </c>
-      <c r="T75" s="6" t="n"/>
+      <c r="S75" s="6" t="n"/>
+      <c r="T75" s="4">
+        <f>IF(COUNT(K75:S75)=0,"",ROUND(SUMPRODUCT(K75:S75,K$4:S$4)/SUM(K$4:S$4),2))</f>
+        <v/>
+      </c>
       <c r="U75" s="6" t="n"/>
+      <c r="V75" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:U75"/>
+  <autoFilter ref="A5:V75"/>
   <mergeCells count="1">
     <mergeCell ref="A2:V2"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D6:D75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Obbligo di legge,Incentivi / fondi,Annunci di lavoro,Recensioni negative,Acquisizioni di verticali,Forum / community,Altro"</formula1>
+      <formula1>"Obbligo di legge,Incentivi / fondi,Annunci di lavoro,Recensioni negative,Acquisizioni di verticali,Forum / community,Ritardi di pagamento,Carenza di manodopera,Dolore operativo permanente,Altro"</formula1>
     </dataValidation>
-    <dataValidation sqref="T6:T75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U6:U75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da studiare,In studio,Da intervistare,Intervistata,Scartata,Scelta"</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:R75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="K6:S75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
@@ -3957,7 +4249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3974,6 +4266,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3986,7 +4279,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Numero di aziende: da fonti dove esistono, altrimenti ipotesi mie, con affidabilità indicata. I PREZZI SONO IPOTESI da validare nelle interviste. Le celle in blu si possono cambiare. 'Quota necessaria' = clienti per 1 M€ diviso aziende target: sopra circa il 10% il mercato italiano è troppo piccolo.</t>
+          <t>Numero di aziende: da fonti dove esistono, altrimenti ipotesi mie, con affidabilità indicata. I PREZZI SONO IPOTESI da validare nelle interviste. Le celle in blu si possono cambiare. 'Quota necessaria' = clienti per 1 M€ diviso aziende target: sopra circa il 10% il mercato italiano è troppo piccolo. 'Bisogno permanente' = 1 se nasce da una scadenza di legge, 5 se è un problema che esiste sempre.</t>
         </is>
       </c>
     </row>
@@ -4113,6 +4406,11 @@
           <t>Lettura</t>
         </is>
       </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Bisogno permanente (1-5, mio giudizio)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -4169,6 +4467,9 @@
           <t>Base ampia, ma mercato affollato di consulenti: serve un canale forte.</t>
         </is>
       </c>
+      <c r="O11" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -4225,6 +4526,9 @@
           <t>Vendi al canale: meno clienti ma con più aziende ciascuno. Da confrontare con le piattaforme esistenti.</t>
         </is>
       </c>
+      <c r="O12" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -4281,6 +4585,9 @@
           <t>Norma europea: il mercato vero è più grande dell'Italia, ma va servito in inglese e con concorrenti internazionali.</t>
         </is>
       </c>
+      <c r="O13" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -4337,6 +4644,9 @@
           <t>Troppo piccolo come solo mercato italiano; ha senso solo come prodotto europeo.</t>
         </is>
       </c>
+      <c r="O14" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -4393,6 +4703,9 @@
           <t>Mercato ben definito e vicino a te; la scadenza (20/01/2027) può slittare.</t>
         </is>
       </c>
+      <c r="O15" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -4449,6 +4762,9 @@
           <t>Tanti utenti ma prezzo basso: serve come aggiunta a un prodotto più grande.</t>
         </is>
       </c>
+      <c r="O16" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -4505,6 +4821,9 @@
           <t>Mercato piccolo e dipendente da pochi committenti.</t>
         </is>
       </c>
+      <c r="O17" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" ht="58" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -4561,6 +4880,9 @@
           <t>Troppo piccolo come mercato solo italiano.</t>
         </is>
       </c>
+      <c r="O18" s="6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="19" ht="58" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -4617,30 +4939,505 @@
           <t>Mercato di nicchia; gli strumenti di misura hanno già report inclusi.</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="O19" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Incassi e solleciti (cassa)</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>45700</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: unità locali con 10+ addetti in ingrosso (46: 20.256), metallo (25: 16.356), macchinari (28: 9.059); basso = 50+ (5.804). Cribis 2026: solo 42% paga puntuale</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J20" s="11">
+        <f>ROUND(1000000/H20,0)</f>
+        <v/>
+      </c>
+      <c r="K20" s="16">
+        <f>J20/C20</f>
+        <v/>
+      </c>
+      <c r="L20" s="17">
+        <f>(1000000/I20)/D20</f>
+        <v/>
+      </c>
+      <c r="M20" s="17">
+        <f>(1000000/G20)/B20</f>
+        <v/>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Bisogno permanente e documentato; concorrenza alta (gestionali e fintech): serve un canale.</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TMS per autotrasporto</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>22700</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 49.41 = 63.633 unità locali, 9.037 con 10+, 915 con 50+; alto = 10+ più 25% delle micro (mia ipotesi). Imprese attive in calo del 22% dal 2015</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Media-bassa</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J21" s="11">
+        <f>ROUND(1000000/H21,0)</f>
+        <v/>
+      </c>
+      <c r="K21" s="16">
+        <f>J21/C21</f>
+        <v/>
+      </c>
+      <c r="L21" s="17">
+        <f>(1000000/I21)/D21</f>
+        <v/>
+      </c>
+      <c r="M21" s="17">
+        <f>(1000000/G21)/B21</f>
+        <v/>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Bisogno permanente, ma il settore si concentra e i clienti diminuiscono.</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Spedizionieri e magazzini</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>850</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>4100</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>6600</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 52.29 e 52.10 con 10+ = 4.123; 50+ = 849; alto = 52.2 con 10+ (6.583)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J22" s="11">
+        <f>ROUND(1000000/H22,0)</f>
+        <v/>
+      </c>
+      <c r="K22" s="16">
+        <f>J22/C22</f>
+        <v/>
+      </c>
+      <c r="L22" s="17">
+        <f>(1000000/I22)/D22</f>
+        <v/>
+      </c>
+      <c r="M22" s="17">
+        <f>(1000000/G22)/B22</f>
+        <v/>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Mercato medio con documenti ripetitivi; concorrenza di software di settore.</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Commesse e tracciabilità (officine)</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>16400</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>25400</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 25 con 10+ = 16.356 (25.62 meccanica generale: 4.975); alto = + 28 con 10+</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J23" s="11">
+        <f>ROUND(1000000/H23,0)</f>
+        <v/>
+      </c>
+      <c r="K23" s="16">
+        <f>J23/C23</f>
+        <v/>
+      </c>
+      <c r="L23" s="17">
+        <f>(1000000/I23)/D23</f>
+        <v/>
+      </c>
+      <c r="M23" s="17">
+        <f>(1000000/G23)/B23</f>
+        <v/>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Quota necessaria bassa, ma serve conoscere il mestiere e ci sono già ERP e MES.</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Preventivatore per distributori tecnici</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: ingrosso di macchinari (466) e prodotti specializzati (467) con 10+ = 8.028; alto = + 25.62 (4.975)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>800</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I24" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J24" s="11">
+        <f>ROUND(1000000/H24,0)</f>
+        <v/>
+      </c>
+      <c r="K24" s="16">
+        <f>J24/C24</f>
+        <v/>
+      </c>
+      <c r="L24" s="17">
+        <f>(1000000/I24)/D24</f>
+        <v/>
+      </c>
+      <c r="M24" s="17">
+        <f>(1000000/G24)/B24</f>
+        <v/>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Legato ai ricavi del cliente; probabili gestionali già presenti, quindi come aggiunta.</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>22700</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: ATECO 28: 9.059 con 10+, 2.179 con 50+, 22.720 totali</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J25" s="11">
+        <f>ROUND(1000000/H25,0)</f>
+        <v/>
+      </c>
+      <c r="K25" s="16">
+        <f>J25/C25</f>
+        <v/>
+      </c>
+      <c r="L25" s="17">
+        <f>(1000000/I25)/D25</f>
+        <v/>
+      </c>
+      <c r="M25" s="17">
+        <f>(1000000/G25)/B25</f>
+        <v/>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Stesso mercato delle macchine, ma bisogno permanente: ogni macchina venduta richiede manuali, ricambi e assistenza per anni.</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Turni per logistica e magazzini</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>850</v>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>4100</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: magazzinaggio e supporto ai trasporti (52) con 10+ = 7.223; 52.10 e 52.29 con 10+ = 4.123</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H26" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I26" s="10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J26" s="11">
+        <f>ROUND(1000000/H26,0)</f>
+        <v/>
+      </c>
+      <c r="K26" s="16">
+        <f>J26/C26</f>
+        <v/>
+      </c>
+      <c r="L26" s="17">
+        <f>(1000000/I26)/D26</f>
+        <v/>
+      </c>
+      <c r="M26" s="17">
+        <f>(1000000/G26)/B26</f>
+        <v/>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Software di turni già diffusi; conta quanto sono complesse le regole del cliente.</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Estrazione dati da ordini e DDT</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>45700</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Istat 2024: come per gli incassi (ingrosso, metallo e macchinari con 10+)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>800</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J27" s="11">
+        <f>ROUND(1000000/H27,0)</f>
+        <v/>
+      </c>
+      <c r="K27" s="16">
+        <f>J27/C27</f>
+        <v/>
+      </c>
+      <c r="L27" s="17">
+        <f>(1000000/I27)/D27</f>
+        <v/>
+      </c>
+      <c r="M27" s="17">
+        <f>(1000000/G27)/B27</f>
+        <v/>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Utile in tutti i settori ma generico: va scelto un solo tipo di documento.</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Come leggerla</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Il numero di aziende viene da Istat 2024 (unità locali, quindi limiti superiori) dove è indicato; le ipotesi residue sono segnate nella colonna Affidabilità. Le norme europee (CRA, RED, Macchine) si applicano in tutta l'UE: il mercato reale può essere molte volte quello italiano, ma richiede un prodotto in inglese e concorrenti internazionali.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Prossimo passo di precisione: il perimetro NIS2 e le quote di prodotti con elementi digitali sono mie approssimazioni, da affinare nelle interviste.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Nessun numero di questo foglio è un dato di mercato verificato per il tuo prodotto: sono ordini di grandezza per scartare le nicchie troppo piccole.</t>
         </is>
@@ -4648,10 +5445,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A23:N23"/>
-    <mergeCell ref="A24:N24"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A22:N22"/>
+    <mergeCell ref="A32:O32"/>
+    <mergeCell ref="A31:O31"/>
+    <mergeCell ref="A30:O30"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
freelance: Fase 3, mappa dei concorrenti, prezzi e canali delle tre finaliste con punteggi provvisori
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNxVApXF9MzdDwSEC8TCy4
</commit_message>
<xml_diff>
--- a/freelance/griglia-nicchie.xlsx
+++ b/freelance/griglia-nicchie.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista lunga" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istat 2024" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 3" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmenti B2B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lista lunga'!$A$5:$V$75</definedName>
@@ -113,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -157,12 +158,16 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1270,15 +1275,33 @@
         <v/>
       </c>
       <c r="J10" s="6" t="n"/>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="6" t="n"/>
-      <c r="P10" s="6" t="n"/>
-      <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="6" t="n"/>
-      <c r="S10" s="6" t="n"/>
+      <c r="K10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="T10" s="4">
         <f>IF(COUNT(K10:S10)=0,"",ROUND(SUMPRODUCT(K10:S10,K$4:S$4)/SUM(K$4:S$4),2))</f>
         <v/>
@@ -2278,15 +2301,33 @@
         <v/>
       </c>
       <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-      <c r="M27" s="6" t="n"/>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="6" t="n"/>
-      <c r="P27" s="6" t="n"/>
-      <c r="Q27" s="6" t="n"/>
-      <c r="R27" s="6" t="n"/>
-      <c r="S27" s="6" t="n"/>
+      <c r="K27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N27" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S27" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="T27" s="4">
         <f>IF(COUNT(K27:S27)=0,"",ROUND(SUMPRODUCT(K27:S27,K$4:S$4)/SUM(K$4:S$4),2))</f>
         <v/>
@@ -2406,15 +2447,33 @@
         <v/>
       </c>
       <c r="J29" s="6" t="n"/>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-      <c r="M29" s="6" t="n"/>
-      <c r="N29" s="6" t="n"/>
-      <c r="O29" s="6" t="n"/>
-      <c r="P29" s="6" t="n"/>
-      <c r="Q29" s="6" t="n"/>
-      <c r="R29" s="6" t="n"/>
-      <c r="S29" s="6" t="n"/>
+      <c r="K29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S29" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="T29" s="4">
         <f>IF(COUNT(K29:S29)=0,"",ROUND(SUMPRODUCT(K29:S29,K$4:S$4)/SUM(K$4:S$4),2))</f>
         <v/>
@@ -2806,15 +2865,33 @@
         <v/>
       </c>
       <c r="J36" s="6" t="n"/>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-      <c r="M36" s="6" t="n"/>
-      <c r="N36" s="6" t="n"/>
-      <c r="O36" s="6" t="n"/>
-      <c r="P36" s="6" t="n"/>
-      <c r="Q36" s="6" t="n"/>
-      <c r="R36" s="6" t="n"/>
-      <c r="S36" s="6" t="n"/>
+      <c r="K36" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M36" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N36" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P36" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S36" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="T36" s="4">
         <f>IF(COUNT(K36:S36)=0,"",ROUND(SUMPRODUCT(K36:S36,K$4:S$4)/SUM(K$4:S$4),2))</f>
         <v/>
@@ -6491,6 +6568,625 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fase 3 — concorrenti, prezzi e canali delle tre finaliste</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Informazioni da siti dei fornitori e stampa, quasi mai da listini ufficiali: i prezzi mancanti sono un risultato, non una dimenticanza. I punteggi nella Lista lunga sono un mio giudizio provvisorio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Finalista</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Concorrente / segnale</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Cosa offre</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Prezzo trovato</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>SYS Suite (Sygest)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Software italiano</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Cataloghi ricambi interattivi 2D/3D, portale web per manuali e offerte, app offline, integrazione ERP/PLM</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>https://www.itismagazine.it/featured/cataloghi-3d-e-interattivi-sys-suite-e-la-soluzione</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Certifico Macchine 4 (CEM4)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Software italiano</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Fascicolo tecnico, archivio norme, check list e valutazione dei rischi per il Regolamento 2023/1230</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>https://www.certifico.com/certifico-macchine-4/manuale-d-uso-ufficiale-di-certifico-macchine-4-cem4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Quanos (cataloghi ricambi)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Software internazionale</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Creazione e pubblicazione di cataloghi ricambi</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>https://quanos.com/en/knowhow/spare-parts-catalog/create-and-publish-spare-parts-catalogs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Salesforce Field Service</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Software per assistenza sul campo</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Gestione interventi e tecnici</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>175 €/utente/mese (230 € versione avanzata), contratto annuale</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com/it/service/field-service-management/pricing/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Dynamics 365 Field Service</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Software per assistenza sul campo</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Gestione interventi e tecnici</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>128,90 $/utente/mese (rivenditore)</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>https://gestisoft.com/en/dynamics-365/field-service</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Altri software di field service</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Mercato</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Panoramica prezzi</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Mediana circa 168 $/utente/mese (intervallo 39-650 $)</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>https://www.costbench.com/software/field-service-management/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Chatbot (RAG) su manuali: nessuna startup italiana trovata</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Lacuna / rischio</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Esistono tesi (IMESA, Padova) e casi internazionali (14.000 tecnici); consulenze su misura possibili</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Non applicabile</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>https://thesis.unipd.it/handle/20.500.12608/95455</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Servizi di manualistica tecnica</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Creazione di manuali e cataloghi ricambi come servizio esterno</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>https://www.reteimprese.it/sers_A105664B100067</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Incassi e solleciti</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Fatture in Cloud (TeamSystem)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Gestionale/fatturazione</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Solleciti automatici di pagamento, anche per importi sopra una soglia</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Da circa 48-60 € + IVA l'anno (fonti discordanti)</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>https://www.fattureincloud.it/software-fatturazione/solleciti-pagamento/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Incassi e solleciti</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Agicap Italia</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Fintech / tesoreria</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Previsione di cassa che raccoglie dati da banche e gestionali; oltre 1.000 clienti in Italia dopo due anni</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>https://www.economyup.it/fintech/fintech-e-pmi-come-agicap-italia-automatizza-la-gestione-dei-flussi-di-cassa/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Incassi e solleciti</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Previxio</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Fintech / tesoreria</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Tesoreria, fatturazione elettronica e previsioni a 12 mesi (da listing non verificato)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>https://www.getapp.com/finance-accounting-software/treasury/f/cash-management/?page=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Incassi e solleciti</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>bexio</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Gestionale (Svizzera)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Solleciti automatici</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>https://www.bexio.com/it-CH/software-fatturazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Preventivatore per distributori tecnici</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Salesforce Revenue Cloud (CPQ)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Configurazione, prezzi e preventivi</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>200 €/utente/mese (fascia Advanced, contratto annuale)</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com/it/products/cpq/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Preventivatore per distributori tecnici</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>ConvertCalculator, iQuoteXpress, Camos CPQ</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>CPQ per PMI / prodotti complessi</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Preventivi configurabili; Camos per prodotti multi-variante</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Non trovato (i costi di implementazione spesso superano il canone)</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>https://www.capterra.it/directory/30904/cpq/software</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Canali di vendita trovati</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>UCIMU: oltre 200 associate (più del 70% del settore, circa 8 miliardi di fatturato); parte di Federmacchine (13 associazioni, tra cui UCIMA)</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>https://www.ucimu.it/en/association/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine)</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Fiere organizzate da Fieramilano: BI-MU, LAMIERA, EMO Milano (date non verificate)</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>https://www.ucimu.it/en/association/ucimu-group/participations/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Sintesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Assistenza post-vendita (macchine): concorrenza frammentata. Software di cataloghi ricambi e di fascicolo tecnico (italiani), field service generico a 130-230 €/utente/mese, nessuna startup italiana trovata sul tema 'assistente AI sui manuali'. Il rischio principale: i costruttori possono costruirsi un RAG da soli con strumenti generici. Il valore deve stare nel flusso di lavoro (ticket, ricambi, multilingue, storico), non nella sola chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Incassi e solleciti: mercato molto presidiato; gli strumenti di fatturazione includono già i solleciti a 50-60 € l'anno e le piattaforme di tesoreria (Agicap, Previxio) coprono la previsione di cassa. Differenziarsi è difficile e il prezzo di riferimento è basso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Preventivatore: i CPQ per aziende grandi costano 200 €/utente/mese; per le PMI non ho trovato listini. Il rischio è di diventare consulenza (ogni cliente richiede configurazione). Un prodotto con importazione automatica di listini potrebbe evitarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Conclusione provvisoria: l'assistenza post-vendita per costruttori di macchine è la candidata principale. Resta da verificare con interviste che il responsabile assistenza abbia il problema e un budget.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId16"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6516,27 +7212,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Segmento</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Quota stimata</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Aziende (stima)</t>
         </is>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Verificato?</t>
         </is>
       </c>
-      <c r="E4" s="21" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Fonte verificata</t>
         </is>
@@ -6548,22 +7244,22 @@
           <t>Manifattura avanzata e meccanica</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>26–28%</t>
         </is>
       </c>
-      <c r="C5" s="22" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>11.000–11.500</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E5" s="24" t="n"/>
+      <c r="E5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="inlineStr">
@@ -6571,22 +7267,22 @@
           <t>Commercio all'ingrosso B2B</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>20–22%</t>
         </is>
       </c>
-      <c r="C6" s="22" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>8.500–9.000</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E6" s="24" t="n"/>
+      <c r="E6" s="27" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
@@ -6594,22 +7290,22 @@
           <t>Servizi corporate, ICT e software</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>12–14%</t>
         </is>
       </c>
-      <c r="C7" s="22" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>5.000–5.800</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E7" s="24" t="n"/>
+      <c r="E7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
@@ -6617,22 +7313,22 @@
           <t>Costruzioni, impiantistica, real estate B2B</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>10–12%</t>
         </is>
       </c>
-      <c r="C8" s="22" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>4.200–4.800</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E8" s="24" t="n"/>
+      <c r="E8" s="27" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
@@ -6640,22 +7336,22 @@
           <t>Chimica, polimeri, gomma-plastica</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>7–8%</t>
         </is>
       </c>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>3.000–3.300</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E9" s="24" t="n"/>
+      <c r="E9" s="27" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
@@ -6663,22 +7359,22 @@
           <t>Logistica, spedizioni e trasporti B2B</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>6–7%</t>
         </is>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>2.500–2.900</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E10" s="24" t="n"/>
+      <c r="E10" s="27" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
@@ -6686,22 +7382,22 @@
           <t>Farmaceutica, biotech, dispositivi medici</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>4–5%</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>1.600–2.000</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E11" s="24" t="n"/>
+      <c r="E11" s="27" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
@@ -6709,22 +7405,22 @@
           <t>Energia, ambiente, utilities B2B</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>3–4%</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>1.300–1.600</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E12" s="24" t="n"/>
+      <c r="E12" s="27" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
@@ -6732,22 +7428,22 @@
           <t>Telecomunicazioni e reti</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>1,5–2%</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>600–800</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E13" s="24" t="n"/>
+      <c r="E13" s="27" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -6788,7 +7484,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6809,7 +7505,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Quasi tutte sono stampa di settore e blog di consulenza, non testi ufficiali: le date vanno confermate sulla fonte primaria.</t>
         </is>
@@ -6821,14 +7517,14 @@
           <t>NIS2</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>https://www.noze.it/insights/nis2-pmi-cyberagent/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/sicurezza/nis2-scadenze-2026-la-guida-per-le-piccole-imprese/</t>
         </is>
@@ -6840,14 +7536,14 @@
           <t>AI Act</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/industry-4-0/digital-omnibus-e-ai-act-cosa-puo-slittare-e-cosa-va-fatto-prima-di-agosto-2026/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>https://www.noze.it/insights/ai-act-digital-omnibus-2026/</t>
         </is>
@@ -6859,14 +7555,14 @@
           <t>Cyber Resilience Act</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/sicurezza/cyber-resilience-act-la-scadenza-chiave-arriva-l11-settembre-2026/</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>https://www.ipsoa.it/documents/quotidiano/2026/09/02/cyber-resilience-act-11-settembre-2026-scatta-obbligo-segnalare-vulnerabilita-incidenti-gravi</t>
         </is>
@@ -6878,14 +7574,14 @@
           <t>Direttiva RED</t>
         </is>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>https://www.tuvsud.com/en-us/services/product-certification/red-cybersecurity-requirements</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>https://www.yarix.com/Advisory-and-Consulting-Services/RED-Compliance</t>
         </is>
@@ -6897,14 +7593,14 @@
           <t>Regolamento Macchine</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>https://certifico.com/macchine/regolamento-ue-2023-1230</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>https://www.ilsussidiario.net/news/regolamento-macchine-ue-rosa-ucimu-mancano-criteri-comuni-e-chiari-serve-una-proroga/2986256/amp/</t>
         </is>
@@ -6916,14 +7612,14 @@
           <t>Trasparenza retributiva</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>https://quifinanza.it/lavoro/trasparenza-salariale-7-giugno-2026/960990/</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>https://www.partitaiva.it/trasparenza-salariale/</t>
         </is>
@@ -6935,7 +7631,7 @@
           <t>PPWR</t>
         </is>
       </c>
-      <c r="B22" s="26" t="inlineStr">
+      <c r="B22" s="23" t="inlineStr">
         <is>
           <t>https://www.assolombarda.it/servizi/ambiente/informazioni/ppwr-dal-12-agosto-in-applicazione-il-nuovo-regolamento-ue-sugli-imballaggi</t>
         </is>
@@ -6947,14 +7643,14 @@
           <t>Passaporto digitale di prodotto</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>https://www.bluestonepim.com/blog/digital-product-passport-for-batteries</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="26" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>https://www.pmi.it/tecnologia/prodotti-e-servizi-ict/492107/passaporto-digitale-prodotto.html</t>
         </is>
@@ -6966,14 +7662,14 @@
           <t>Accessibilità (EAA)</t>
         </is>
       </c>
-      <c r="B27" s="26" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/mercati-digitali/ecommerce/siti-ecommerce-accessibili-guida-in-5-step-per-evitare-sanzioni/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="26" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>https://www.iubenda.com/it/help/178476-accessibilita-101/</t>
         </is>
@@ -6985,14 +7681,14 @@
           <t>Iperammortamento 2026</t>
         </is>
       </c>
-      <c r="B30" s="26" t="inlineStr">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>https://www.agendadigitale.eu/industry-4-0/iperammortamento-2026-la-guida-cose-e-come-fare-le-comunicazioni-al-gse/</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="26" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>https://pasqualepillitteri.it/perizia-iperammortamento</t>
         </is>
@@ -7004,7 +7700,7 @@
           <t>Acquisizioni TeamSystem / Zucchetti</t>
         </is>
       </c>
-      <c r="B33" s="26" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>https://aventis-advisors.com/teamsystem-acquisitions/</t>
         </is>
@@ -7016,14 +7712,14 @@
           <t>Piano Italia 1 Giga</t>
         </is>
       </c>
-      <c r="B35" s="26" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t>https://www.editorialedomani.it/economia/banda-ultralarga-cantieri-obiettivi-pnrr-ritardi-regioni-oqbs3i02</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="26" t="inlineStr">
+      <c r="B36" s="23" t="inlineStr">
         <is>
           <t>https://tariffe.segugio.it/news-tariffe/italia-1-giga-nuovi-ritardi-per-la-banda-ultra-larga-cosa-sta-succedendo-00043657.aspx</t>
         </is>
@@ -7035,14 +7731,14 @@
           <t>FWA e frequenze 26 GHz</t>
         </is>
       </c>
-      <c r="B38" s="26" t="inlineStr">
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t>https://tariffe.segugio.it/news-tariffe/internet-senza-fibra-la-fwa-supera-2-7-milioni-di-linee-00047779.aspx</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="26" t="inlineStr">
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t>https://www.smartworld.it/news/frequenze-5g-26-ghz-gara-italia-agosto-2026.html</t>
         </is>
@@ -7054,42 +7750,42 @@
           <t>Fase 2 — numeri di mercato</t>
         </is>
       </c>
-      <c r="B41" s="26" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://esploradati.istat.it (dataset: Classe di addetti, settori economici (Ateco 5 cifre) - Italia, anno 2024)</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="26" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://accredia.it/wp-content/uploads/2024/07/Cartella-stampa-breve-dati-al-31-12-2025_ITA-1.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="26" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://assomac.it/media/documents/rapporto_federmacchine_2020.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="26" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>https://anie.it/federazione/chi-siamo/rapporto-annuale-2025_def</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="26" t="inlineStr">
+      <c r="B45" s="23" t="inlineStr">
         <is>
           <t>https://www.cni.it/images/eventi/2021/01_Lelaborazione_delle_perizie_13lug2021.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="26" t="inlineStr">
+      <c r="B46" s="23" t="inlineStr">
         <is>
           <t>https://www.fibertelecom.com/wt/2022/PDF/02-puglia/FTWWT2022-puglia-03.pdf</t>
         </is>
@@ -7101,7 +7797,7 @@
           <t>Comunità energetiche (CER)</t>
         </is>
       </c>
-      <c r="B48" s="26" t="inlineStr">
+      <c r="B48" s="23" t="inlineStr">
         <is>
           <t>https://www.infobuildenergia.it/approfondimenti/cer-comunita-energetiche-in-italia/</t>
         </is>

</xml_diff>